<commit_message>
📊 Horarios actualizados Línea 141 - 2162
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-03.xlsx
+++ b/data/horarios-141-2026-04-03.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:02:38</t>
+          <t>Última actualización: 02:46:41</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 2</t>
+          <t>Total filas: 3</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>01:02:38</t>
+          <t>02:46:41</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>01:25</t>
+          <t>03:01</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,23 +498,48 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>01:02:38</t>
+          <t>02:46:41</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>03:01</t>
+          <t>03:48</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>119</v>
+        <v>62</v>
       </c>
       <c r="E7" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>02:46:41</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>04:02</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>76</v>
+      </c>
+      <c r="E8" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -544,7 +569,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:02:38</t>
+          <t>Última actualización: 02:46:41</t>
         </is>
       </c>
     </row>
@@ -579,7 +604,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:02:38</t>
+          <t>Última actualización: 02:46:41</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2163
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-03.xlsx
+++ b/data/horarios-141-2026-04-03.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:46:41</t>
+          <t>Última actualización: 03:51:10</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 3</t>
+          <t>Total filas: 8</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>02:46:41</t>
+          <t>03:51:10</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>03:01</t>
+          <t>03:51</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>02:46:41</t>
+          <t>03:51:10</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>03:48</t>
+          <t>04:02</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>62</v>
+        <v>11</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,12 +523,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>02:46:41</t>
+          <t>03:51:10</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>04:02</t>
+          <t>04:48</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -537,9 +537,134 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>76</v>
+        <v>57</v>
       </c>
       <c r="E8" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>03:51:10</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>04:53</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>62</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>03:51:10</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>05:17</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>86</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>03:51:10</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>05:22</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>91</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>03:51:10</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>05:47</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>116</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>03:51:10</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>05:47</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>116</v>
+      </c>
+      <c r="E13" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -569,7 +694,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:46:41</t>
+          <t>Última actualización: 03:51:10</t>
         </is>
       </c>
     </row>
@@ -604,7 +729,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:46:41</t>
+          <t>Última actualización: 03:51:10</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2164
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-03.xlsx
+++ b/data/horarios-141-2026-04-03.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:51:10</t>
+          <t>Última actualización: 04:54:42</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 8</t>
+          <t>Total filas: 13</t>
         </is>
       </c>
     </row>
@@ -473,17 +473,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>03:51:10</t>
+          <t>04:54:42</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>03:51</t>
+          <t>04:54</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>03:51:10</t>
+          <t>04:54:42</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>04:02</t>
+          <t>05:17</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,21 +523,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>03:51:10</t>
+          <t>04:54:42</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>04:48</t>
+          <t>05:22</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>57</v>
+        <v>28</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -548,21 +548,21 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>03:51:10</t>
+          <t>04:54:42</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>04:53</t>
+          <t>05:44</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>62</v>
+        <v>50</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -573,21 +573,21 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>03:51:10</t>
+          <t>04:54:42</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>05:17</t>
+          <t>05:46</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>86</v>
+        <v>52</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -598,21 +598,21 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>03:51:10</t>
+          <t>04:54:42</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>05:22</t>
+          <t>06:01</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>91</v>
+        <v>67</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -623,21 +623,21 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>03:51:10</t>
+          <t>04:54:42</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>05:47</t>
+          <t>06:09</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>116</v>
+        <v>75</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -648,23 +648,148 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>03:51:10</t>
+          <t>04:54:42</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>05:47</t>
+          <t>06:12</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>116</v>
+        <v>78</v>
       </c>
       <c r="E13" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>04:54:42</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>06:30</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>96</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>04:54:42</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>06:36</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>102</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>04:54:42</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>06:39</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>105</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>04:54:42</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>06:40</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>106</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>04:54:42</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>06:41</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>107</v>
+      </c>
+      <c r="E18" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -681,7 +806,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -694,14 +819,66 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:51:10</t>
+          <t>Última actualización: 04:54:42</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 0</t>
+          <t>Total filas: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Hora_Scrap</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Hora_Llegada</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Linea</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Minutos</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Parada</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>04:54:42</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>06:12</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>78</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>LP1912</t>
         </is>
       </c>
     </row>
@@ -729,7 +906,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:51:10</t>
+          <t>Última actualización: 04:54:42</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2165
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-03.xlsx
+++ b/data/horarios-141-2026-04-03.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:54:42</t>
+          <t>Última actualización: 05:40:21</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 13</t>
+          <t>Total filas: 17</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>04:54:42</t>
+          <t>05:40:21</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>04:54</t>
+          <t>05:41</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>04:54:42</t>
+          <t>05:40:21</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>05:17</t>
+          <t>05:47</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>23</v>
+        <v>7</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,21 +523,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>04:54:42</t>
+          <t>05:40:21</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>05:22</t>
+          <t>06:09</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -548,21 +548,21 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>04:54:42</t>
+          <t>05:40:21</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>05:44</t>
+          <t>06:12</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>50</v>
+        <v>32</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -573,21 +573,21 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>04:54:42</t>
+          <t>05:40:21</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>05:46</t>
+          <t>06:30</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -598,21 +598,21 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>04:54:42</t>
+          <t>05:40:21</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>06:01</t>
+          <t>06:36</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>67</v>
+        <v>56</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -623,21 +623,21 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>04:54:42</t>
+          <t>05:40:21</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>06:09</t>
+          <t>06:39</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -648,21 +648,21 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>04:54:42</t>
+          <t>05:40:21</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>06:12</t>
+          <t>06:41</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>78</v>
+        <v>61</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -673,21 +673,21 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>04:54:42</t>
+          <t>05:40:21</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>06:41</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>96</v>
+        <v>61</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -698,21 +698,21 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>04:54:42</t>
+          <t>05:40:21</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>06:36</t>
+          <t>06:59</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>102</v>
+        <v>79</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -723,21 +723,21 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>04:54:42</t>
+          <t>05:40:21</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>06:39</t>
+          <t>07:02</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>105</v>
+        <v>82</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,12 +748,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>04:54:42</t>
+          <t>05:40:21</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>06:40</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -762,7 +762,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -773,23 +773,123 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>04:54:42</t>
+          <t>05:40:21</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>06:41</t>
+          <t>07:26</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D18" t="n">
+        <v>106</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>05:40:21</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>07:27</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
         <v>107</v>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>05:40:21</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>07:32</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>112</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>05:40:21</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>07:37</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>117</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>05:40:21</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>07:37</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>117</v>
+      </c>
+      <c r="E22" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -806,7 +906,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -819,14 +919,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:54:42</t>
+          <t>Última actualización: 05:40:21</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 1</t>
+          <t>Total filas: 3</t>
         </is>
       </c>
     </row>
@@ -860,7 +960,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>04:54:42</t>
+          <t>05:40:21</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -874,9 +974,59 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>78</v>
+        <v>32</v>
       </c>
       <c r="E6" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>05:40:21</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>07:02</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>82</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>05:40:21</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>07:32</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>112</v>
+      </c>
+      <c r="E8" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -906,7 +1056,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:54:42</t>
+          <t>Última actualización: 05:40:21</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2166
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-03.xlsx
+++ b/data/horarios-141-2026-04-03.xlsx
@@ -432,7 +432,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:40:21</t>
+          <t>Última actualización: 06:36:21</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>05:40:21</t>
+          <t>06:36:21</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>05:41</t>
+          <t>06:36</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>05:40:21</t>
+          <t>06:36:21</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>05:47</t>
+          <t>06:39</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,21 +523,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>05:40:21</t>
+          <t>06:36:21</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>06:09</t>
+          <t>06:41</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>29</v>
+        <v>5</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -548,21 +548,21 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>05:40:21</t>
+          <t>06:36:21</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>06:12</t>
+          <t>06:41</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>32</v>
+        <v>5</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -573,21 +573,21 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>05:40:21</t>
+          <t>06:36:21</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>06:59</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>50</v>
+        <v>23</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -598,21 +598,21 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>05:40:21</t>
+          <t>06:36:21</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>06:36</t>
+          <t>07:02</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>56</v>
+        <v>26</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -623,21 +623,21 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>05:40:21</t>
+          <t>06:36:21</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>06:39</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>59</v>
+        <v>45</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -648,21 +648,21 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>05:40:21</t>
+          <t>06:36:21</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>06:41</t>
+          <t>07:26</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>61</v>
+        <v>50</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -673,21 +673,21 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>05:40:21</t>
+          <t>06:36:21</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>06:41</t>
+          <t>07:27</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -698,21 +698,21 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>05:40:21</t>
+          <t>06:36:21</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>06:59</t>
+          <t>07:32</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>79</v>
+        <v>56</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -723,21 +723,21 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>05:40:21</t>
+          <t>06:36:21</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>07:02</t>
+          <t>07:37</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>82</v>
+        <v>61</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,21 +748,21 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>05:40:21</t>
+          <t>06:36:21</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>07:21</t>
+          <t>07:44</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>101</v>
+        <v>68</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -773,21 +773,21 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>05:40:21</t>
+          <t>06:36:21</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>07:26</t>
+          <t>07:51</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>106</v>
+        <v>75</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -798,12 +798,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>05:40:21</t>
+          <t>06:36:21</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>07:27</t>
+          <t>08:06</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -812,7 +812,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>107</v>
+        <v>90</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -823,21 +823,21 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>05:40:21</t>
+          <t>06:36:21</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>07:32</t>
+          <t>08:19</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>112</v>
+        <v>103</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -848,21 +848,21 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>05:40:21</t>
+          <t>06:36:21</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>07:37</t>
+          <t>08:21</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>117</v>
+        <v>105</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -873,21 +873,21 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>05:40:21</t>
+          <t>06:36:21</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>07:37</t>
+          <t>08:26</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -919,7 +919,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:40:21</t>
+          <t>Última actualización: 06:36:21</t>
         </is>
       </c>
     </row>
@@ -960,12 +960,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>05:40:21</t>
+          <t>06:36:21</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>06:12</t>
+          <t>07:02</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -974,7 +974,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -985,21 +985,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>05:40:21</t>
+          <t>06:36:21</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>07:02</t>
+          <t>07:32</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>82</v>
+        <v>56</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -1010,21 +1010,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>05:40:21</t>
+          <t>06:36:21</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>07:32</t>
+          <t>07:51</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>112</v>
+        <v>75</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -1043,7 +1043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1056,14 +1056,66 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:40:21</t>
+          <t>Última actualización: 06:36:21</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 0</t>
+          <t>Total filas: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Hora_Scrap</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Hora_Llegada</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Linea</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Minutos</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Parada</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>06:36:21</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>07:49</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>73</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2167
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-03.xlsx
+++ b/data/horarios-141-2026-04-03.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:36:21</t>
+          <t>Última actualización: 07:22:46</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 17</t>
+          <t>Total filas: 28</t>
         </is>
       </c>
     </row>
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -558,7 +558,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -648,7 +648,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>06:36:21</t>
+          <t>07:22:46</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -662,7 +662,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>50</v>
+        <v>4</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -673,7 +673,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>06:36:21</t>
+          <t>07:22:46</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -687,7 +687,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>51</v>
+        <v>5</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -698,12 +698,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>06:36:21</t>
+          <t>07:22:46</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>07:32</t>
+          <t>07:31</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -712,7 +712,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>56</v>
+        <v>9</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -728,16 +728,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>07:37</t>
+          <t>07:32</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,21 +748,21 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>06:36:21</t>
+          <t>07:22:46</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>07:44</t>
+          <t>07:36</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>68</v>
+        <v>14</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -778,16 +778,16 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>07:51</t>
+          <t>07:37</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>75</v>
+        <v>61</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -798,21 +798,21 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>06:36:21</t>
+          <t>07:22:46</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>08:06</t>
+          <t>07:44</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>90</v>
+        <v>22</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -823,21 +823,21 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>06:36:21</t>
+          <t>07:22:46</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>08:19</t>
+          <t>07:51</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>103</v>
+        <v>29</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -848,21 +848,21 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>06:36:21</t>
+          <t>07:22:46</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>08:21</t>
+          <t>08:01</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>105</v>
+        <v>39</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -873,23 +873,298 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t>07:22:46</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>08:06</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>44</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>07:22:46</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>08:19</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>57</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
           <t>06:36:21</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>08:21</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>105</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>07:22:46</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>08:25</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>63</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>06:36:21</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
         <is>
           <t>08:26</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D22" t="n">
+      <c r="D26" t="n">
         <v>110</v>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>07:22:46</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>08:44</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>82</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>07:22:46</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>08:44</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>82</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>07:22:46</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>09:04</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>102</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>07:22:46</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>09:05</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>103</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>07:22:46</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>09:06</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>104</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>07:22:46</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>09:16</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>114</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>07:22:46</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>09:16</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>114</v>
+      </c>
+      <c r="E33" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -906,7 +1181,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -919,14 +1194,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:36:21</t>
+          <t>Última actualización: 07:22:46</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 3</t>
+          <t>Total filas: 7</t>
         </is>
       </c>
     </row>
@@ -985,12 +1260,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>06:36:21</t>
+          <t>07:22:46</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>07:32</t>
+          <t>07:31</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -999,7 +1274,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>56</v>
+        <v>9</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -1015,18 +1290,118 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
+          <t>07:32</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>56</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>07:22:46</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
           <t>07:51</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D8" t="n">
-        <v>75</v>
-      </c>
-      <c r="E8" t="inlineStr">
+      <c r="D9" t="n">
+        <v>29</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>07:22:46</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>08:44</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>82</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>07:22:46</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>08:44</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>82</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>07:22:46</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>09:06</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>104</v>
+      </c>
+      <c r="E12" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1043,7 +1418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1056,14 +1431,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:36:21</t>
+          <t>Última actualización: 07:22:46</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 1</t>
+          <t>Total filas: 4</t>
         </is>
       </c>
     </row>
@@ -1097,25 +1472,100 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>07:22:46</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>07:48</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>26</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
           <t>06:36:21</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>07:49</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D6" t="n">
+      <c r="D7" t="n">
         <v>73</v>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>07:22:46</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>08:37</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>75</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>07:22:46</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>09:02</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>100</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2168
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-03.xlsx
+++ b/data/horarios-141-2026-04-03.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:22:46</t>
+          <t>Última actualización: 08:07:05</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 28</t>
+          <t>Total filas: 39</t>
         </is>
       </c>
     </row>
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -558,7 +558,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -898,7 +898,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>07:22:46</t>
+          <t>08:07:05</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -912,7 +912,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>57</v>
+        <v>12</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -948,21 +948,21 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>07:22:46</t>
+          <t>08:07:05</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>08:25</t>
+          <t>08:24</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>63</v>
+        <v>17</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -973,12 +973,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>06:36:21</t>
+          <t>07:22:46</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>08:26</t>
+          <t>08:25</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -987,7 +987,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>110</v>
+        <v>63</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -998,21 +998,21 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>07:22:46</t>
+          <t>08:07:05</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>08:44</t>
+          <t>08:26</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>82</v>
+        <v>19</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1023,21 +1023,21 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>07:22:46</t>
+          <t>08:07:05</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>08:44</t>
+          <t>08:42</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>82</v>
+        <v>35</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1053,16 +1053,16 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>09:04</t>
+          <t>08:44</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>102</v>
+        <v>82</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1078,16 +1078,16 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>09:05</t>
+          <t>08:44</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>103</v>
+        <v>82</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1098,21 +1098,21 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>07:22:46</t>
+          <t>08:07:05</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>09:06</t>
+          <t>08:45</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>104</v>
+        <v>38</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1123,21 +1123,21 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>07:22:46</t>
+          <t>08:07:05</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>09:16</t>
+          <t>08:45</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>114</v>
+        <v>38</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1148,23 +1148,298 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
+          <t>08:07:05</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>09:04</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>57</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>08:07:05</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>09:05</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>58</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
           <t>07:22:46</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>09:06</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>104</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>08:07:05</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>09:07</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>60</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>07:22:46</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
         <is>
           <t>09:16</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C37" t="inlineStr">
         <is>
           <t>27_EL RETIRO</t>
         </is>
       </c>
-      <c r="D33" t="n">
+      <c r="D37" t="n">
         <v>114</v>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>08:07:05</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>09:16</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>69</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>08:07:05</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>09:17</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>70</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>08:07:05</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>09:24</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>77</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>08:07:05</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>09:35</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>88</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>08:07:05</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>09:45</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>98</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>08:07:05</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>09:55</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>108</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>08:07:05</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>09:59</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>112</v>
+      </c>
+      <c r="E44" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1181,7 +1456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1194,14 +1469,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:22:46</t>
+          <t>Última actualización: 08:07:05</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 7</t>
+          <t>Total filas: 11</t>
         </is>
       </c>
     </row>
@@ -1385,23 +1660,123 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>08:07:05</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>08:45</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>38</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>08:07:05</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>08:45</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>38</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>07:22:46</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>09:06</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D12" t="n">
+      <c r="D14" t="n">
         <v>104</v>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>08:07:05</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>09:07</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>60</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>08:07:05</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>09:55</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>108</v>
+      </c>
+      <c r="E16" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1418,7 +1793,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1431,14 +1806,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:22:46</t>
+          <t>Última actualización: 08:07:05</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 4</t>
+          <t>Total filas: 7</t>
         </is>
       </c>
     </row>
@@ -1547,25 +1922,100 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>08:07:05</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>08:38</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>31</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>07:22:46</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>09:02</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D9" t="n">
+      <c r="D10" t="n">
         <v>100</v>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>08:07:05</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>09:03</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>56</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>08:07:05</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>09:28</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>81</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2169
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-03.xlsx
+++ b/data/horarios-141-2026-04-03.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:E55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:07:05</t>
+          <t>Última actualización: 08:49:34</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 39</t>
+          <t>Total filas: 50</t>
         </is>
       </c>
     </row>
@@ -1148,21 +1148,21 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>08:07:05</t>
+          <t>08:49:34</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>09:04</t>
+          <t>08:49</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>57</v>
+        <v>0</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1173,21 +1173,21 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>08:07:05</t>
+          <t>08:49:34</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>09:05</t>
+          <t>09:04</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>58</v>
+        <v>15</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1198,21 +1198,21 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>07:22:46</t>
+          <t>08:07:05</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>09:06</t>
+          <t>09:05</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>104</v>
+        <v>58</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1223,12 +1223,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>08:07:05</t>
+          <t>08:49:34</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>09:07</t>
+          <t>09:06</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1237,7 +1237,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>60</v>
+        <v>17</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1248,21 +1248,21 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>07:22:46</t>
+          <t>08:07:05</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>09:16</t>
+          <t>09:07</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>114</v>
+        <v>60</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1273,21 +1273,21 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>08:07:05</t>
+          <t>08:49:34</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>09:16</t>
+          <t>09:11</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>69</v>
+        <v>22</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1298,12 +1298,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>08:07:05</t>
+          <t>08:49:34</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>09:17</t>
+          <t>09:16</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1312,7 +1312,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1323,21 +1323,21 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>08:07:05</t>
+          <t>08:49:34</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>09:24</t>
+          <t>09:16</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>77</v>
+        <v>27</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1353,16 +1353,16 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>09:35</t>
+          <t>09:17</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1373,21 +1373,21 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>08:07:05</t>
+          <t>08:49:34</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>09:45</t>
+          <t>09:24</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>98</v>
+        <v>35</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,21 +1398,21 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>08:07:05</t>
+          <t>08:49:34</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>09:55</t>
+          <t>09:35</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>108</v>
+        <v>46</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1423,23 +1423,298 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
+          <t>08:49:34</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>09:44</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>55</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
           <t>08:07:05</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr">
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>09:45</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>98</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>08:49:34</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>09:51</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>62</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>08:49:34</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>09:55</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>66</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>08:49:34</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>09:58</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>69</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>08:07:05</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
         <is>
           <t>09:59</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
+      <c r="C49" t="inlineStr">
         <is>
           <t>10_OLMOS</t>
         </is>
       </c>
-      <c r="D44" t="n">
+      <c r="D49" t="n">
         <v>112</v>
       </c>
-      <c r="E44" t="inlineStr">
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>08:49:34</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>10:05</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>76</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>08:49:34</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>10:15</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>86</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>08:49:34</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>10:24</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>95</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>08:49:34</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>10:34</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>105</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>08:49:34</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>10:39</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>110</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>08:49:34</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>10:44</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>115</v>
+      </c>
+      <c r="E55" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1456,7 +1731,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1469,14 +1744,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:07:05</t>
+          <t>Última actualización: 08:49:34</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 11</t>
+          <t>Total filas: 12</t>
         </is>
       </c>
     </row>
@@ -1710,21 +1985,21 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>07:22:46</t>
+          <t>08:49:34</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>09:06</t>
+          <t>08:49</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>104</v>
+        <v>0</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -1735,12 +2010,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>08:07:05</t>
+          <t>08:49:34</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>09:07</t>
+          <t>09:06</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1749,7 +2024,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>60</v>
+        <v>17</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -1765,18 +2040,43 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
+          <t>09:07</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>60</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>08:49:34</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
           <t>09:55</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D16" t="n">
-        <v>108</v>
-      </c>
-      <c r="E16" t="inlineStr">
+      <c r="D17" t="n">
+        <v>66</v>
+      </c>
+      <c r="E17" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1793,7 +2093,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1806,14 +2106,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:07:05</t>
+          <t>Última actualización: 08:49:34</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 7</t>
+          <t>Total filas: 10</t>
         </is>
       </c>
     </row>
@@ -1947,7 +2247,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>07:22:46</t>
+          <t>08:49:34</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1961,7 +2261,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>100</v>
+        <v>13</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -1997,7 +2297,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>08:07:05</t>
+          <t>08:49:34</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -2011,9 +2311,84 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>81</v>
+        <v>39</v>
       </c>
       <c r="E12" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>08:49:34</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>10:17</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>88</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>08:49:34</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>101</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>08:49:34</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>10:43</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>114</v>
+      </c>
+      <c r="E15" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2170
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-03.xlsx
+++ b/data/horarios-141-2026-04-03.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E55"/>
+  <dimension ref="A1:E67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:49:34</t>
+          <t>Última actualización: 09:30:27</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 50</t>
+          <t>Total filas: 62</t>
         </is>
       </c>
     </row>
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -558,7 +558,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -1058,7 +1058,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D29" t="n">
@@ -1083,7 +1083,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D30" t="n">
@@ -1398,21 +1398,21 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>08:49:34</t>
+          <t>09:30:27</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>09:35</t>
+          <t>09:34</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>46</v>
+        <v>4</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1423,21 +1423,21 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>08:49:34</t>
+          <t>09:30:27</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>09:44</t>
+          <t>09:35</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>55</v>
+        <v>5</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,12 +1448,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>08:07:05</t>
+          <t>09:30:27</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>09:45</t>
+          <t>09:44</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1462,7 +1462,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>98</v>
+        <v>14</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1473,21 +1473,21 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>08:49:34</t>
+          <t>08:07:05</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>09:51</t>
+          <t>09:45</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>62</v>
+        <v>98</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1498,21 +1498,21 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>08:49:34</t>
+          <t>09:30:27</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>09:55</t>
+          <t>09:51</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>66</v>
+        <v>21</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1523,21 +1523,21 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>08:49:34</t>
+          <t>09:30:27</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>09:58</t>
+          <t>09:55</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>69</v>
+        <v>25</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1548,12 +1548,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>08:07:05</t>
+          <t>08:49:34</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>09:59</t>
+          <t>09:58</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -1562,7 +1562,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>112</v>
+        <v>69</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1573,21 +1573,21 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>08:49:34</t>
+          <t>08:07:05</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>10:05</t>
+          <t>09:59</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>76</v>
+        <v>112</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1598,21 +1598,21 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>08:49:34</t>
+          <t>09:30:27</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>10:15</t>
+          <t>10:01</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>86</v>
+        <v>31</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1623,21 +1623,21 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>08:49:34</t>
+          <t>09:30:27</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>10:24</t>
+          <t>10:04</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>95</v>
+        <v>34</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -1653,16 +1653,16 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>10:34</t>
+          <t>10:05</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>105</v>
+        <v>76</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -1673,21 +1673,21 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>08:49:34</t>
+          <t>09:30:27</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>10:39</t>
+          <t>10:10</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>110</v>
+        <v>40</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1698,23 +1698,323 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
+          <t>09:30:27</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>10:15</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>45</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>09:30:27</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>10:24</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>54</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>09:30:27</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>10:34</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>64</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
           <t>08:49:34</t>
         </is>
       </c>
-      <c r="B55" t="inlineStr">
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>10:39</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>110</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>09:30:27</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
         <is>
           <t>10:44</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr">
+      <c r="C59" t="inlineStr">
         <is>
           <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D55" t="n">
-        <v>115</v>
-      </c>
-      <c r="E55" t="inlineStr">
+      <c r="D59" t="n">
+        <v>74</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>09:30:27</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>10:48</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>78</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>09:30:27</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>10:53</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>83</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>09:30:27</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>10:55</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>85</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>09:30:27</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>11:01</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>91</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>09:30:27</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>11:04</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>94</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>09:30:27</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>11:08</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>98</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>09:30:27</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>11:15</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>105</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>09:30:27</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>11:24</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>114</v>
+      </c>
+      <c r="E67" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1744,7 +2044,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:49:34</t>
+          <t>Última actualización: 09:30:27</t>
         </is>
       </c>
     </row>
@@ -2060,7 +2360,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>08:49:34</t>
+          <t>09:30:27</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2074,7 +2374,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>66</v>
+        <v>25</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -2093,7 +2393,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2106,14 +2406,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:49:34</t>
+          <t>Última actualización: 09:30:27</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 10</t>
+          <t>Total filas: 13</t>
         </is>
       </c>
     </row>
@@ -2322,25 +2622,25 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>08:49:34</t>
+          <t>09:30:27</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>10:17</t>
+          <t>09:30</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>215C_LA PLATA</t>
+          <t>215A_LA PLATA</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>88</v>
+        <v>0</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>L6203</t>
+          <t>L6173</t>
         </is>
       </c>
     </row>
@@ -2352,45 +2652,120 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10:30</t>
+          <t>10:17</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>215B_LP-P MOR-1 Y 57</t>
+          <t>215C_LA PLATA</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>101</v>
+        <v>88</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>L6173</t>
+          <t>L6203</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>08:49:34</t>
+          <t>09:30:27</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
+          <t>10:18</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>48</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>09:30:27</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>60</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>09:30:27</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
           <t>10:43</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D15" t="n">
-        <v>114</v>
-      </c>
-      <c r="E15" t="inlineStr">
+      <c r="D17" t="n">
+        <v>73</v>
+      </c>
+      <c r="E17" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>09:30:27</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>11:23</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>113</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2171
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-03.xlsx
+++ b/data/horarios-141-2026-04-03.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E67"/>
+  <dimension ref="A1:E81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:30:27</t>
+          <t>Última actualización: 10:46:22</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 62</t>
+          <t>Total filas: 76</t>
         </is>
       </c>
     </row>
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -558,7 +558,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -1058,7 +1058,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D29" t="n">
@@ -1083,7 +1083,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D30" t="n">
@@ -1108,7 +1108,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D31" t="n">
@@ -1133,7 +1133,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1333,7 +1333,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -1848,21 +1848,21 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>09:30:27</t>
+          <t>10:46:22</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>10:53</t>
+          <t>10:51</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>83</v>
+        <v>5</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1878,16 +1878,16 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>10:55</t>
+          <t>10:53</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1898,21 +1898,21 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>09:30:27</t>
+          <t>10:46:22</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>11:01</t>
+          <t>10:55</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>91</v>
+        <v>9</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1923,21 +1923,21 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>09:30:27</t>
+          <t>10:46:22</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>11:04</t>
+          <t>10:57</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>94</v>
+        <v>11</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1948,21 +1948,21 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>09:30:27</t>
+          <t>10:46:22</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>11:08</t>
+          <t>11:01</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>98</v>
+        <v>15</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1973,21 +1973,21 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>09:30:27</t>
+          <t>10:46:22</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>11:15</t>
+          <t>11:04</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>105</v>
+        <v>18</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -1998,23 +1998,373 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>09:30:27</t>
+          <t>10:46:22</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
+          <t>11:08</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>22</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>10:46:22</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>11:15</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>29</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>10:46:22</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
           <t>11:24</t>
         </is>
       </c>
-      <c r="C67" t="inlineStr">
+      <c r="C69" t="inlineStr">
         <is>
           <t>10_OLMOS</t>
         </is>
       </c>
-      <c r="D67" t="n">
-        <v>114</v>
-      </c>
-      <c r="E67" t="inlineStr">
+      <c r="D69" t="n">
+        <v>38</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>10:46:22</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>11:35</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>49</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>10:46:22</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>11:36</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>50</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>10:46:22</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>11:39</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>53</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>10:46:22</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>11:44</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>58</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>10:46:22</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>11:54</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>68</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>10:46:22</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>11:55</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>69</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>10:46:22</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>12:04</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>78</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>10:46:22</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>89</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>10:46:22</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>12:24</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>98</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>10:46:22</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>12:34</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>108</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>10:46:22</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>12:37</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>111</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>10:46:22</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>12:44</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>118</v>
+      </c>
+      <c r="E81" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2031,7 +2381,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2044,14 +2394,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:30:27</t>
+          <t>Última actualización: 10:46:22</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 12</t>
+          <t>Total filas: 14</t>
         </is>
       </c>
     </row>
@@ -2377,6 +2727,56 @@
         <v>25</v>
       </c>
       <c r="E17" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>10:46:22</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>11:35</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>49</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>10:46:22</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>11:44</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>58</v>
+      </c>
+      <c r="E19" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2406,7 +2806,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:30:27</t>
+          <t>Última actualización: 10:46:22</t>
         </is>
       </c>
     </row>
@@ -2747,7 +3147,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>09:30:27</t>
+          <t>10:46:22</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2761,7 +3161,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>113</v>
+        <v>37</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2172
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-03.xlsx
+++ b/data/horarios-141-2026-04-03.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E81"/>
+  <dimension ref="A1:E91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:46:22</t>
+          <t>Última actualización: 11:28:49</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 76</t>
+          <t>Total filas: 86</t>
         </is>
       </c>
     </row>
@@ -1108,7 +1108,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D31" t="n">
@@ -1133,7 +1133,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -2073,12 +2073,12 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>10:46:22</t>
+          <t>11:28:49</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>11:35</t>
+          <t>11:34</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -2087,7 +2087,7 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>49</v>
+        <v>6</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2103,16 +2103,16 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>11:36</t>
+          <t>11:35</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2123,21 +2123,21 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>10:46:22</t>
+          <t>11:28:49</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>11:39</t>
+          <t>11:36</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>53</v>
+        <v>8</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -2153,16 +2153,16 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>11:44</t>
+          <t>11:39</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2173,21 +2173,21 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>10:46:22</t>
+          <t>11:28:49</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>11:54</t>
+          <t>11:41</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>68</v>
+        <v>13</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2198,21 +2198,21 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>10:46:22</t>
+          <t>11:28:49</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>11:55</t>
+          <t>11:44</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>69</v>
+        <v>16</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2223,21 +2223,21 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>10:46:22</t>
+          <t>11:28:49</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>12:04</t>
+          <t>11:54</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>78</v>
+        <v>26</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2248,21 +2248,21 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>10:46:22</t>
+          <t>11:28:49</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>12:15</t>
+          <t>11:55</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>89</v>
+        <v>27</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2273,21 +2273,21 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>10:46:22</t>
+          <t>11:28:49</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>12:24</t>
+          <t>12:04</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>98</v>
+        <v>36</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2298,21 +2298,21 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>10:46:22</t>
+          <t>11:28:49</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>12:34</t>
+          <t>12:15</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>108</v>
+        <v>47</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -2323,21 +2323,21 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>10:46:22</t>
+          <t>11:28:49</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>12:37</t>
+          <t>12:24</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>111</v>
+        <v>56</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2348,23 +2348,273 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
+          <t>11:28:49</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>62</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>11:28:49</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>12:32</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>64</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>11:28:49</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>12:34</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>66</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
           <t>10:46:22</t>
         </is>
       </c>
-      <c r="B81" t="inlineStr">
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>12:37</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>111</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>11:28:49</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>12:43</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>75</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>10:46:22</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
         <is>
           <t>12:44</t>
         </is>
       </c>
-      <c r="C81" t="inlineStr">
+      <c r="C86" t="inlineStr">
         <is>
           <t>14X44_ABASTO</t>
         </is>
       </c>
-      <c r="D81" t="n">
+      <c r="D86" t="n">
         <v>118</v>
       </c>
-      <c r="E81" t="inlineStr">
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>11:28:49</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>12:46</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>78</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>11:28:49</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>12:54</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>86</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>11:28:49</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>13:04</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>96</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>11:28:49</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>107</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>11:28:49</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>13:24</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>116</v>
+      </c>
+      <c r="E91" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2381,7 +2631,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2394,14 +2644,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:46:22</t>
+          <t>Última actualización: 11:28:49</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 14</t>
+          <t>Total filas: 16</t>
         </is>
       </c>
     </row>
@@ -2545,7 +2795,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -2570,7 +2820,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -2595,7 +2845,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -2620,7 +2870,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -2735,12 +2985,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>10:46:22</t>
+          <t>11:28:49</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>11:35</t>
+          <t>11:34</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2749,7 +2999,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>49</v>
+        <v>6</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -2765,18 +3015,68 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
+          <t>11:35</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>49</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>11:28:49</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
           <t>11:44</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>215B_EL PATO</t>
         </is>
       </c>
-      <c r="D19" t="n">
-        <v>58</v>
-      </c>
-      <c r="E19" t="inlineStr">
+      <c r="D20" t="n">
+        <v>16</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>11:28:49</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>12:54</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>86</v>
+      </c>
+      <c r="E21" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2793,7 +3093,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2806,14 +3106,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:46:22</t>
+          <t>Última actualización: 11:28:49</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 13</t>
+          <t>Total filas: 14</t>
         </is>
       </c>
     </row>
@@ -3164,6 +3464,31 @@
         <v>37</v>
       </c>
       <c r="E18" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>11:28:49</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>13:22</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>114</v>
+      </c>
+      <c r="E19" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2173
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-03.xlsx
+++ b/data/horarios-141-2026-04-03.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E91"/>
+  <dimension ref="A1:E99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:28:49</t>
+          <t>Última actualización: 12:08:20</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 86</t>
+          <t>Total filas: 94</t>
         </is>
       </c>
     </row>
@@ -1058,7 +1058,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D29" t="n">
@@ -1083,7 +1083,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D30" t="n">
@@ -1108,7 +1108,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D31" t="n">
@@ -1133,7 +1133,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1333,7 +1333,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -2298,21 +2298,21 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>11:28:49</t>
+          <t>12:08:20</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>12:15</t>
+          <t>12:08</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>47</v>
+        <v>0</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -2323,21 +2323,21 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>11:28:49</t>
+          <t>12:08:20</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>12:24</t>
+          <t>12:15</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>56</v>
+        <v>7</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2348,21 +2348,21 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>11:28:49</t>
+          <t>12:08:20</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>12:30</t>
+          <t>12:24</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>62</v>
+        <v>16</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2378,16 +2378,16 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>12:32</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2398,21 +2398,21 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>11:28:49</t>
+          <t>12:08:20</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>12:34</t>
+          <t>12:31</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>66</v>
+        <v>23</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2423,21 +2423,21 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>10:46:22</t>
+          <t>11:28:49</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>12:37</t>
+          <t>12:32</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>111</v>
+        <v>64</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2448,21 +2448,21 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>11:28:49</t>
+          <t>12:08:20</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>12:43</t>
+          <t>12:34</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>75</v>
+        <v>26</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -2473,21 +2473,21 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>10:46:22</t>
+          <t>12:08:20</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>12:44</t>
+          <t>12:37</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>118</v>
+        <v>29</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2503,16 +2503,16 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>12:46</t>
+          <t>12:43</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2523,21 +2523,21 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>11:28:49</t>
+          <t>12:08:20</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>12:54</t>
+          <t>12:44</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>86</v>
+        <v>36</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2548,21 +2548,21 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>11:28:49</t>
+          <t>12:08:20</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>13:04</t>
+          <t>12:46</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>96</v>
+        <v>38</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -2578,16 +2578,16 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>13:15</t>
+          <t>12:54</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>107</v>
+        <v>86</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2598,23 +2598,223 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>11:28:49</t>
+          <t>12:08:20</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
+          <t>12:55</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>47</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>12:08:20</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>13:04</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>56</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>12:08:20</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>67</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>12:08:20</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
           <t>13:24</t>
         </is>
       </c>
-      <c r="C91" t="inlineStr">
+      <c r="C94" t="inlineStr">
         <is>
           <t>10_OLMOS</t>
         </is>
       </c>
-      <c r="D91" t="n">
+      <c r="D94" t="n">
+        <v>76</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>12:08:20</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>13:26</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>78</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>12:08:20</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>13:31</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>83</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>12:08:20</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>13:44</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D97" t="n">
+        <v>96</v>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>12:08:20</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>13:55</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D98" t="n">
+        <v>107</v>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>12:08:20</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>14:04</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D99" t="n">
         <v>116</v>
       </c>
-      <c r="E91" t="inlineStr">
+      <c r="E99" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2631,7 +2831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2644,14 +2844,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:28:49</t>
+          <t>Última actualización: 12:08:20</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 16</t>
+          <t>Total filas: 18</t>
         </is>
       </c>
     </row>
@@ -3077,6 +3277,56 @@
         <v>86</v>
       </c>
       <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>12:08:20</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>12:55</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>47</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>12:08:20</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>13:31</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>83</v>
+      </c>
+      <c r="E23" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3093,7 +3343,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3106,14 +3356,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:28:49</t>
+          <t>Última actualización: 12:08:20</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 14</t>
+          <t>Total filas: 16</t>
         </is>
       </c>
     </row>
@@ -3491,6 +3741,56 @@
       <c r="E19" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>12:08:20</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>13:23</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>75</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>12:08:20</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>13:50</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>102</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2174
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-03.xlsx
+++ b/data/horarios-141-2026-04-03.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E99"/>
+  <dimension ref="A1:E109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:08:20</t>
+          <t>Última actualización: 12:51:38</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 94</t>
+          <t>Total filas: 104</t>
         </is>
       </c>
     </row>
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -558,7 +558,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -1058,7 +1058,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D29" t="n">
@@ -1083,7 +1083,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D30" t="n">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1333,7 +1333,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -2573,7 +2573,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>11:28:49</t>
+          <t>12:51:38</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -2587,7 +2587,7 @@
         </is>
       </c>
       <c r="D90" t="n">
-        <v>86</v>
+        <v>3</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2623,7 +2623,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>12:08:20</t>
+          <t>12:51:38</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2637,7 +2637,7 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>56</v>
+        <v>13</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2648,7 +2648,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>12:08:20</t>
+          <t>12:51:38</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -2662,7 +2662,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>67</v>
+        <v>24</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -2673,21 +2673,21 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>12:08:20</t>
+          <t>12:51:38</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>13:24</t>
+          <t>13:21</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>76</v>
+        <v>30</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2698,21 +2698,21 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>12:08:20</t>
+          <t>12:51:38</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>13:26</t>
+          <t>13:24</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>78</v>
+        <v>33</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2728,16 +2728,16 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>13:31</t>
+          <t>13:26</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2748,21 +2748,21 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>12:08:20</t>
+          <t>12:51:38</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>13:44</t>
+          <t>13:31</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>96</v>
+        <v>40</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2773,21 +2773,21 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>12:08:20</t>
+          <t>12:51:38</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>13:55</t>
+          <t>13:44</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>107</v>
+        <v>53</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2798,23 +2798,273 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>12:08:20</t>
+          <t>12:51:38</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
+          <t>13:55</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D99" t="n">
+        <v>64</v>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>12:51:38</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>13:56</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D100" t="n">
+        <v>65</v>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>12:51:38</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
           <t>14:04</t>
         </is>
       </c>
-      <c r="C99" t="inlineStr">
+      <c r="C101" t="inlineStr">
         <is>
           <t>225_GOMEZ</t>
         </is>
       </c>
-      <c r="D99" t="n">
-        <v>116</v>
-      </c>
-      <c r="E99" t="inlineStr">
+      <c r="D101" t="n">
+        <v>73</v>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>12:51:38</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>14:11</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D102" t="n">
+        <v>80</v>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>12:51:38</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>14:14</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D103" t="n">
+        <v>83</v>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>12:51:38</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>14:14</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D104" t="n">
+        <v>83</v>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>12:51:38</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>14:16</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D105" t="n">
+        <v>85</v>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>12:51:38</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>14:24</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D106" t="n">
+        <v>93</v>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>12:51:38</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>14:31</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D107" t="n">
+        <v>100</v>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>12:51:38</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>14:34</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D108" t="n">
+        <v>103</v>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>12:51:38</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>14:44</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D109" t="n">
+        <v>113</v>
+      </c>
+      <c r="E109" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2831,7 +3081,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2844,14 +3094,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:08:20</t>
+          <t>Última actualización: 12:51:38</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 18</t>
+          <t>Total filas: 19</t>
         </is>
       </c>
     </row>
@@ -3260,7 +3510,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>11:28:49</t>
+          <t>12:51:38</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -3274,7 +3524,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>86</v>
+        <v>3</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -3310,7 +3560,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>12:08:20</t>
+          <t>12:51:38</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -3324,9 +3574,34 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>83</v>
+        <v>40</v>
       </c>
       <c r="E23" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>12:51:38</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>14:34</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>103</v>
+      </c>
+      <c r="E24" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3343,7 +3618,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3356,14 +3631,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:08:20</t>
+          <t>Última actualización: 12:51:38</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 16</t>
+          <t>Total filas: 18</t>
         </is>
       </c>
     </row>
@@ -3722,7 +3997,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>11:28:49</t>
+          <t>12:51:38</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -3736,7 +4011,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>114</v>
+        <v>31</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -3772,25 +4047,75 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>12:51:38</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>13:49</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>58</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
           <t>12:08:20</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>13:50</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-1 Y 57</t>
         </is>
       </c>
-      <c r="D21" t="n">
+      <c r="D22" t="n">
         <v>102</v>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="E22" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>12:51:38</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>14:42</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>111</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2175
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-03.xlsx
+++ b/data/horarios-141-2026-04-03.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E109"/>
+  <dimension ref="A1:E122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:51:38</t>
+          <t>Última actualización: 13:27:06</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 104</t>
+          <t>Total filas: 117</t>
         </is>
       </c>
     </row>
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -558,7 +558,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1333,7 +1333,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -2773,21 +2773,21 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>12:51:38</t>
+          <t>13:27:06</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>13:44</t>
+          <t>13:32</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>53</v>
+        <v>5</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2803,16 +2803,16 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>13:55</t>
+          <t>13:44</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>64</v>
+        <v>53</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -2823,21 +2823,21 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>12:51:38</t>
+          <t>13:27:06</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>13:56</t>
+          <t>13:45</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>65</v>
+        <v>18</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -2848,21 +2848,21 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>12:51:38</t>
+          <t>13:27:06</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>14:04</t>
+          <t>13:55</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>73</v>
+        <v>28</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -2878,16 +2878,16 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>14:11</t>
+          <t>13:56</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>80</v>
+        <v>65</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2898,21 +2898,21 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>12:51:38</t>
+          <t>13:27:06</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>14:14</t>
+          <t>14:04</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>83</v>
+        <v>37</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -2928,16 +2928,16 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>14:14</t>
+          <t>14:11</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -2948,21 +2948,21 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>12:51:38</t>
+          <t>13:27:06</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>14:16</t>
+          <t>14:12</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>85</v>
+        <v>45</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -2973,21 +2973,21 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>12:51:38</t>
+          <t>13:27:06</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>14:24</t>
+          <t>14:14</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>93</v>
+        <v>47</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -2998,21 +2998,21 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>12:51:38</t>
+          <t>13:27:06</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>14:31</t>
+          <t>14:14</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>100</v>
+        <v>47</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3028,16 +3028,16 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>14:34</t>
+          <t>14:16</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>103</v>
+        <v>85</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -3048,23 +3048,348 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
+          <t>13:27:06</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>14:17</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D109" t="n">
+        <v>50</v>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
           <t>12:51:38</t>
         </is>
       </c>
-      <c r="B109" t="inlineStr">
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>14:24</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D110" t="n">
+        <v>93</v>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>13:27:06</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>14:25</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D111" t="n">
+        <v>58</v>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>12:51:38</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>14:31</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D112" t="n">
+        <v>100</v>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>12:51:38</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>14:34</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D113" t="n">
+        <v>103</v>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>13:27:06</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>14:35</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D114" t="n">
+        <v>68</v>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>13:27:06</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>14:35</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D115" t="n">
+        <v>68</v>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>13:27:06</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
         <is>
           <t>14:44</t>
         </is>
       </c>
-      <c r="C109" t="inlineStr">
+      <c r="C116" t="inlineStr">
         <is>
           <t>10_OLMOS</t>
         </is>
       </c>
-      <c r="D109" t="n">
-        <v>113</v>
-      </c>
-      <c r="E109" t="inlineStr">
+      <c r="D116" t="n">
+        <v>77</v>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>13:27:06</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>14:55</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D117" t="n">
+        <v>88</v>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>13:27:06</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D118" t="n">
+        <v>93</v>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>13:27:06</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>15:05</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D119" t="n">
+        <v>98</v>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>13:27:06</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>15:07</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D120" t="n">
+        <v>100</v>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>13:27:06</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>15:15</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D121" t="n">
+        <v>108</v>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>13:27:06</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>15:24</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D122" t="n">
+        <v>117</v>
+      </c>
+      <c r="E122" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3081,7 +3406,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3094,14 +3419,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:51:38</t>
+          <t>Última actualización: 13:27:06</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 19</t>
+          <t>Total filas: 23</t>
         </is>
       </c>
     </row>
@@ -3585,23 +3910,123 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>13:27:06</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>13:32</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>5</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
           <t>12:51:38</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>14:34</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D24" t="n">
+      <c r="D25" t="n">
         <v>103</v>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>13:27:06</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>14:35</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>68</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>13:27:06</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>14:55</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>88</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>13:27:06</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>15:05</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>98</v>
+      </c>
+      <c r="E28" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3618,7 +4043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3631,14 +4056,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:51:38</t>
+          <t>Última actualización: 13:27:06</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 18</t>
+          <t>Total filas: 21</t>
         </is>
       </c>
     </row>
@@ -4047,37 +4472,37 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>12:51:38</t>
+          <t>13:27:06</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>13:49</t>
+          <t>13:27</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>215B_LP-P MOR-1 Y 57</t>
+          <t>215C_LA PLATA</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>58</v>
+        <v>0</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>L6173</t>
+          <t>L6203</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>12:08:20</t>
+          <t>12:51:38</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>13:50</t>
+          <t>13:49</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -4086,7 +4511,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>102</v>
+        <v>58</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -4097,25 +4522,100 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t>13:27:06</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>13:50</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>23</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
           <t>12:51:38</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>14:42</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D23" t="n">
+      <c r="D24" t="n">
         <v>111</v>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="E24" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>13:27:06</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>14:43</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>76</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>13:27:06</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>15:23</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>116</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2176
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-03.xlsx
+++ b/data/horarios-141-2026-04-03.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E122"/>
+  <dimension ref="A1:E135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:27:06</t>
+          <t>Última actualización: 14:01:59</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 117</t>
+          <t>Total filas: 130</t>
         </is>
       </c>
     </row>
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -558,7 +558,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -1058,7 +1058,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D29" t="n">
@@ -1083,7 +1083,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D30" t="n">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1333,7 +1333,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -2898,12 +2898,12 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>13:27:06</t>
+          <t>14:01:59</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>14:04</t>
+          <t>14:03</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -2912,7 +2912,7 @@
         </is>
       </c>
       <c r="D103" t="n">
-        <v>37</v>
+        <v>2</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -2923,21 +2923,21 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>12:51:38</t>
+          <t>13:27:06</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>14:11</t>
+          <t>14:04</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>80</v>
+        <v>37</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -2948,12 +2948,12 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>13:27:06</t>
+          <t>14:01:59</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>14:12</t>
+          <t>14:11</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -2962,7 +2962,7 @@
         </is>
       </c>
       <c r="D105" t="n">
-        <v>45</v>
+        <v>10</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -2978,16 +2978,16 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>14:14</t>
+          <t>14:12</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -2998,7 +2998,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>13:27:06</t>
+          <t>14:01:59</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -3012,7 +3012,7 @@
         </is>
       </c>
       <c r="D107" t="n">
-        <v>47</v>
+        <v>13</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3023,21 +3023,21 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>12:51:38</t>
+          <t>14:01:59</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>14:16</t>
+          <t>14:14</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>85</v>
+        <v>13</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -3048,12 +3048,12 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>13:27:06</t>
+          <t>14:01:59</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>14:17</t>
+          <t>14:16</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -3062,7 +3062,7 @@
         </is>
       </c>
       <c r="D109" t="n">
-        <v>50</v>
+        <v>15</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,21 +3073,21 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>12:51:38</t>
+          <t>13:27:06</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>14:24</t>
+          <t>14:17</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>93</v>
+        <v>50</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3098,12 +3098,12 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>13:27:06</t>
+          <t>14:01:59</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>14:25</t>
+          <t>14:24</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -3112,7 +3112,7 @@
         </is>
       </c>
       <c r="D111" t="n">
-        <v>58</v>
+        <v>23</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -3123,21 +3123,21 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>12:51:38</t>
+          <t>13:27:06</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>14:31</t>
+          <t>14:25</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>100</v>
+        <v>58</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -3153,16 +3153,16 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>14:34</t>
+          <t>14:31</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D113" t="n">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
@@ -3173,21 +3173,21 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>13:27:06</t>
+          <t>14:01:59</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>14:35</t>
+          <t>14:34</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>68</v>
+        <v>33</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3208,7 +3208,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D115" t="n">
@@ -3228,16 +3228,16 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>14:44</t>
+          <t>14:35</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>77</v>
+        <v>68</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3248,21 +3248,21 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>13:27:06</t>
+          <t>14:01:59</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>14:55</t>
+          <t>14:36</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>88</v>
+        <v>35</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -3273,21 +3273,21 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>13:27:06</t>
+          <t>14:01:59</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>14:43</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D118" t="n">
-        <v>93</v>
+        <v>42</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -3303,16 +3303,16 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>15:05</t>
+          <t>14:44</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D119" t="n">
-        <v>98</v>
+        <v>77</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
@@ -3323,21 +3323,21 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>13:27:06</t>
+          <t>14:01:59</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>15:07</t>
+          <t>14:54</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>100</v>
+        <v>53</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3353,16 +3353,16 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>15:15</t>
+          <t>14:55</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>108</v>
+        <v>88</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3373,23 +3373,348 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
+          <t>14:01:59</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>14:57</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D122" t="n">
+        <v>56</v>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
           <t>13:27:06</t>
         </is>
       </c>
-      <c r="B122" t="inlineStr">
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D123" t="n">
+        <v>93</v>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>14:01:59</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>15:04</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D124" t="n">
+        <v>63</v>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>13:27:06</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>15:05</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D125" t="n">
+        <v>98</v>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>14:01:59</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>15:06</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D126" t="n">
+        <v>65</v>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>13:27:06</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>15:07</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D127" t="n">
+        <v>100</v>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>14:01:59</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>15:15</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D128" t="n">
+        <v>74</v>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>14:01:59</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>15:23</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D129" t="n">
+        <v>82</v>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>13:27:06</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
         <is>
           <t>15:24</t>
         </is>
       </c>
-      <c r="C122" t="inlineStr">
+      <c r="C130" t="inlineStr">
         <is>
           <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D122" t="n">
+      <c r="D130" t="n">
         <v>117</v>
       </c>
-      <c r="E122" t="inlineStr">
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>14:01:59</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>15:34</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D131" t="n">
+        <v>93</v>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>14:01:59</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>15:44</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D132" t="n">
+        <v>103</v>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>14:01:59</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>15:55</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D133" t="n">
+        <v>114</v>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>14:01:59</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>15:55</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D134" t="n">
+        <v>114</v>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>14:01:59</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>15:56</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D135" t="n">
+        <v>115</v>
+      </c>
+      <c r="E135" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3406,7 +3731,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3419,14 +3744,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:27:06</t>
+          <t>Última actualización: 14:01:59</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 23</t>
+          <t>Total filas: 26</t>
         </is>
       </c>
     </row>
@@ -3935,7 +4260,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>12:51:38</t>
+          <t>14:01:59</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -3949,7 +4274,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>103</v>
+        <v>33</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -3985,12 +4310,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>13:27:06</t>
+          <t>14:01:59</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>14:55</t>
+          <t>14:54</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -3999,7 +4324,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>88</v>
+        <v>53</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -4015,18 +4340,93 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
+          <t>14:55</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>88</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>14:01:59</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>15:04</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>63</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>13:27:06</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
           <t>15:05</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>215B_EL PATO</t>
         </is>
       </c>
-      <c r="D28" t="n">
+      <c r="D30" t="n">
         <v>98</v>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>14:01:59</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>15:34</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>93</v>
+      </c>
+      <c r="E31" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4043,7 +4443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4056,14 +4456,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:27:06</t>
+          <t>Última actualización: 14:01:59</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 21</t>
+          <t>Total filas: 22</t>
         </is>
       </c>
     </row>
@@ -4547,7 +4947,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>12:51:38</t>
+          <t>14:01:59</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -4561,7 +4961,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>111</v>
+        <v>41</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -4597,23 +4997,48 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
+          <t>14:01:59</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>15:22</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>81</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
           <t>13:27:06</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
           <t>15:23</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D26" t="n">
+      <c r="D27" t="n">
         <v>116</v>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="E27" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2177
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-03.xlsx
+++ b/data/horarios-141-2026-04-03.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E135"/>
+  <dimension ref="A1:E146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:01:59</t>
+          <t>Última actualización: 14:48:24</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 130</t>
+          <t>Total filas: 141</t>
         </is>
       </c>
     </row>
@@ -1108,7 +1108,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D31" t="n">
@@ -1133,7 +1133,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1333,7 +1333,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -3008,7 +3008,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -3033,7 +3033,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D108" t="n">
@@ -3348,7 +3348,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>13:27:06</t>
+          <t>14:48:24</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -3362,7 +3362,7 @@
         </is>
       </c>
       <c r="D121" t="n">
-        <v>88</v>
+        <v>7</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3448,21 +3448,21 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>13:27:06</t>
+          <t>14:48:24</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>15:05</t>
+          <t>15:04</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>98</v>
+        <v>16</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,21 +3473,21 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>14:01:59</t>
+          <t>14:48:24</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>15:06</t>
+          <t>15:05</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>65</v>
+        <v>17</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3498,12 +3498,12 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>13:27:06</t>
+          <t>14:48:24</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>15:07</t>
+          <t>15:06</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -3512,7 +3512,7 @@
         </is>
       </c>
       <c r="D127" t="n">
-        <v>100</v>
+        <v>18</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3523,21 +3523,21 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>14:01:59</t>
+          <t>13:27:06</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>15:15</t>
+          <t>15:07</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>74</v>
+        <v>100</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,21 +3548,21 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>14:01:59</t>
+          <t>14:48:24</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>15:23</t>
+          <t>15:15</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>82</v>
+        <v>27</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3573,12 +3573,12 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>13:27:06</t>
+          <t>14:01:59</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>15:24</t>
+          <t>15:23</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
@@ -3587,7 +3587,7 @@
         </is>
       </c>
       <c r="D130" t="n">
-        <v>117</v>
+        <v>82</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -3598,21 +3598,21 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>14:01:59</t>
+          <t>14:48:24</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>15:34</t>
+          <t>15:24</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>93</v>
+        <v>36</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3628,16 +3628,16 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>15:44</t>
+          <t>15:34</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,21 +3648,21 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>14:01:59</t>
+          <t>14:48:24</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>15:55</t>
+          <t>15:35</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>114</v>
+        <v>47</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3673,21 +3673,21 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>14:01:59</t>
+          <t>14:48:24</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>15:55</t>
+          <t>15:41</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D134" t="n">
-        <v>114</v>
+        <v>53</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -3698,23 +3698,298 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
+          <t>14:48:24</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>15:44</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D135" t="n">
+        <v>56</v>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>14:48:24</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>15:53</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D136" t="n">
+        <v>65</v>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>14:48:24</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>15:55</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D137" t="n">
+        <v>67</v>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
           <t>14:01:59</t>
         </is>
       </c>
-      <c r="B135" t="inlineStr">
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>15:55</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D138" t="n">
+        <v>114</v>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>14:01:59</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
         <is>
           <t>15:56</t>
         </is>
       </c>
-      <c r="C135" t="inlineStr">
+      <c r="C139" t="inlineStr">
         <is>
           <t>27_EL RETIRO</t>
         </is>
       </c>
-      <c r="D135" t="n">
+      <c r="D139" t="n">
         <v>115</v>
       </c>
-      <c r="E135" t="inlineStr">
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>14:48:24</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>15:57</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D140" t="n">
+        <v>69</v>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>14:48:24</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>16:04</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D141" t="n">
+        <v>76</v>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>14:48:24</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>16:14</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D142" t="n">
+        <v>86</v>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>14:48:24</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>16:24</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D143" t="n">
+        <v>96</v>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>14:48:24</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>16:34</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D144" t="n">
+        <v>106</v>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>14:48:24</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>16:35</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D145" t="n">
+        <v>107</v>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>14:48:24</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>16:44</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D146" t="n">
+        <v>116</v>
+      </c>
+      <c r="E146" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3731,7 +4006,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3744,14 +4019,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:01:59</t>
+          <t>Última actualización: 14:48:24</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 26</t>
+          <t>Total filas: 27</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4610,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>13:27:06</t>
+          <t>14:48:24</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -4349,7 +4624,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>88</v>
+        <v>7</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -4385,7 +4660,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>13:27:06</t>
+          <t>14:48:24</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -4399,7 +4674,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>98</v>
+        <v>17</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -4427,6 +4702,31 @@
         <v>93</v>
       </c>
       <c r="E31" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>14:48:24</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>15:35</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>47</v>
+      </c>
+      <c r="E32" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4443,7 +4743,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4456,14 +4756,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:01:59</t>
+          <t>Última actualización: 14:48:24</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 22</t>
+          <t>Total filas: 24</t>
         </is>
       </c>
     </row>
@@ -5022,7 +5322,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>13:27:06</t>
+          <t>14:48:24</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -5036,9 +5336,59 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>116</v>
+        <v>35</v>
       </c>
       <c r="E27" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>14:48:24</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>16:03</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>75</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>14:48:24</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>102</v>
+      </c>
+      <c r="E29" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2178
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-03.xlsx
+++ b/data/horarios-141-2026-04-03.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E146"/>
+  <dimension ref="A1:E154"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:48:24</t>
+          <t>Última actualización: 15:25:49</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 141</t>
+          <t>Total filas: 149</t>
         </is>
       </c>
     </row>
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -558,7 +558,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -1058,7 +1058,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D29" t="n">
@@ -1083,7 +1083,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D30" t="n">
@@ -1108,7 +1108,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D31" t="n">
@@ -1133,7 +1133,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -3623,21 +3623,21 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>14:01:59</t>
+          <t>15:25:49</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>15:34</t>
+          <t>15:25</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>93</v>
+        <v>0</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,12 +3648,12 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>14:48:24</t>
+          <t>15:25:49</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>15:35</t>
+          <t>15:34</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
@@ -3662,7 +3662,7 @@
         </is>
       </c>
       <c r="D133" t="n">
-        <v>47</v>
+        <v>9</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3678,16 +3678,16 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>15:41</t>
+          <t>15:35</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D134" t="n">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -3698,21 +3698,21 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>14:48:24</t>
+          <t>15:25:49</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>15:44</t>
+          <t>15:41</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D135" t="n">
-        <v>56</v>
+        <v>16</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -3723,21 +3723,21 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>14:48:24</t>
+          <t>15:25:49</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>15:53</t>
+          <t>15:44</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>65</v>
+        <v>19</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,21 +3748,21 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>14:48:24</t>
+          <t>15:25:49</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>15:55</t>
+          <t>15:51</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>67</v>
+        <v>26</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3773,21 +3773,21 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>14:01:59</t>
+          <t>14:48:24</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>15:55</t>
+          <t>15:53</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>114</v>
+        <v>65</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3803,16 +3803,16 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>15:56</t>
+          <t>15:55</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D139" t="n">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -3823,21 +3823,21 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>14:48:24</t>
+          <t>15:25:49</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>15:57</t>
+          <t>15:55</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D140" t="n">
-        <v>69</v>
+        <v>30</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
@@ -3848,21 +3848,21 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>14:48:24</t>
+          <t>15:25:49</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>16:04</t>
+          <t>15:56</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D141" t="n">
-        <v>76</v>
+        <v>31</v>
       </c>
       <c r="E141" t="inlineStr">
         <is>
@@ -3878,16 +3878,16 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>16:14</t>
+          <t>15:57</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D142" t="n">
-        <v>86</v>
+        <v>69</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3898,21 +3898,21 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>14:48:24</t>
+          <t>15:25:49</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>16:24</t>
+          <t>16:04</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>96</v>
+        <v>39</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3923,21 +3923,21 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>14:48:24</t>
+          <t>15:25:49</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>16:34</t>
+          <t>16:14</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>106</v>
+        <v>49</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -3948,21 +3948,21 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>14:48:24</t>
+          <t>15:25:49</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>16:35</t>
+          <t>16:24</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D145" t="n">
-        <v>107</v>
+        <v>59</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3973,23 +3973,223 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>14:48:24</t>
+          <t>15:25:49</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
+          <t>16:32</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D146" t="n">
+        <v>67</v>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>15:25:49</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>16:34</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D147" t="n">
+        <v>69</v>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>15:25:49</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>16:35</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D148" t="n">
+        <v>70</v>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>15:25:49</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>16:41</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D149" t="n">
+        <v>76</v>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>15:25:49</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
           <t>16:44</t>
         </is>
       </c>
-      <c r="C146" t="inlineStr">
+      <c r="C150" t="inlineStr">
         <is>
           <t>225_GOMEZ</t>
         </is>
       </c>
-      <c r="D146" t="n">
-        <v>116</v>
-      </c>
-      <c r="E146" t="inlineStr">
+      <c r="D150" t="n">
+        <v>79</v>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>15:25:49</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>16:55</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D151" t="n">
+        <v>90</v>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>15:25:49</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>17:04</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D152" t="n">
+        <v>99</v>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>15:25:49</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>17:14</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D153" t="n">
+        <v>109</v>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>15:25:49</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>17:24</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D154" t="n">
+        <v>119</v>
+      </c>
+      <c r="E154" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4006,7 +4206,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4019,14 +4219,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:48:24</t>
+          <t>Última actualización: 15:25:49</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 27</t>
+          <t>Total filas: 28</t>
         </is>
       </c>
     </row>
@@ -4685,7 +4885,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>14:01:59</t>
+          <t>15:25:49</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -4699,7 +4899,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>93</v>
+        <v>9</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -4727,6 +4927,31 @@
         <v>47</v>
       </c>
       <c r="E32" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>15:25:49</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>17:14</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>109</v>
+      </c>
+      <c r="E33" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4743,7 +4968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4756,14 +4981,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:48:24</t>
+          <t>Última actualización: 15:25:49</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 24</t>
+          <t>Total filas: 28</t>
         </is>
       </c>
     </row>
@@ -5347,50 +5572,150 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>14:48:24</t>
+          <t>15:25:49</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>16:03</t>
+          <t>15:26</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>215C_LA PLATA</t>
+          <t>215A_LA PLATA</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>75</v>
+        <v>1</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>L6203</t>
+          <t>L6173</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
+          <t>15:25:49</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>16:02</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>37</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
           <t>14:48:24</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>16:03</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>75</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>15:25:49</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>16:29</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>64</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>14:48:24</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
         <is>
           <t>16:30</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-40 Y 115</t>
         </is>
       </c>
-      <c r="D29" t="n">
+      <c r="D32" t="n">
         <v>102</v>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="E32" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>15:25:49</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>17:22</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>117</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2179
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-03.xlsx
+++ b/data/horarios-141-2026-04-03.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E154"/>
+  <dimension ref="A1:E166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:25:49</t>
+          <t>Última actualización: 16:09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 149</t>
+          <t>Total filas: 161</t>
         </is>
       </c>
     </row>
@@ -1108,7 +1108,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D31" t="n">
@@ -1133,7 +1133,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -3008,7 +3008,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -3033,7 +3033,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D108" t="n">
@@ -3208,7 +3208,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D115" t="n">
@@ -3233,7 +3233,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D116" t="n">
@@ -3798,7 +3798,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>14:01:59</t>
+          <t>15:25:49</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -3808,11 +3808,11 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D139" t="n">
-        <v>114</v>
+        <v>30</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -3823,7 +3823,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>15:25:49</t>
+          <t>14:01:59</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -3833,11 +3833,11 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D140" t="n">
-        <v>30</v>
+        <v>114</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
@@ -3923,7 +3923,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>15:25:49</t>
+          <t>16:09:00</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -3937,7 +3937,7 @@
         </is>
       </c>
       <c r="D144" t="n">
-        <v>49</v>
+        <v>5</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -3948,21 +3948,21 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>15:25:49</t>
+          <t>16:09:00</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>16:24</t>
+          <t>16:22</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D145" t="n">
-        <v>59</v>
+        <v>13</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3978,16 +3978,16 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>16:32</t>
+          <t>16:24</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -3998,21 +3998,21 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>15:25:49</t>
+          <t>16:09:00</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>16:34</t>
+          <t>16:25</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D147" t="n">
-        <v>69</v>
+        <v>16</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -4028,16 +4028,16 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>16:35</t>
+          <t>16:32</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4048,21 +4048,21 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>15:25:49</t>
+          <t>16:09:00</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>16:41</t>
+          <t>16:34</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D149" t="n">
-        <v>76</v>
+        <v>25</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -4073,21 +4073,21 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>15:25:49</t>
+          <t>16:09:00</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>16:44</t>
+          <t>16:35</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D150" t="n">
-        <v>79</v>
+        <v>26</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -4103,16 +4103,16 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>16:55</t>
+          <t>16:41</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D151" t="n">
-        <v>90</v>
+        <v>76</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -4123,21 +4123,21 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>15:25:49</t>
+          <t>16:09:00</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>17:04</t>
+          <t>16:42</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>99</v>
+        <v>33</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,21 +4148,21 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>15:25:49</t>
+          <t>16:09:00</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>17:14</t>
+          <t>16:44</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>109</v>
+        <v>35</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4173,23 +4173,323 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
+          <t>16:09:00</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>16:51</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D154" t="n">
+        <v>42</v>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>16:09:00</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>16:55</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D155" t="n">
+        <v>46</v>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
           <t>15:25:49</t>
         </is>
       </c>
-      <c r="B154" t="inlineStr">
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>17:04</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D156" t="n">
+        <v>99</v>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>16:09:00</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>17:05</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D157" t="n">
+        <v>56</v>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>15:25:49</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>17:14</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D158" t="n">
+        <v>109</v>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>16:09:00</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>17:15</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D159" t="n">
+        <v>66</v>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>16:09:00</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
         <is>
           <t>17:24</t>
         </is>
       </c>
-      <c r="C154" t="inlineStr">
+      <c r="C160" t="inlineStr">
         <is>
           <t>10_OLMOS</t>
         </is>
       </c>
-      <c r="D154" t="n">
+      <c r="D160" t="n">
+        <v>75</v>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>16:09:00</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>17:34</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D161" t="n">
+        <v>85</v>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>16:09:00</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>17:35</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D162" t="n">
+        <v>86</v>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>16:09:00</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>17:38</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D163" t="n">
+        <v>89</v>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>16:09:00</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>17:45</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D164" t="n">
+        <v>96</v>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>16:09:00</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>17:55</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D165" t="n">
+        <v>106</v>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>16:09:00</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>18:08</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D166" t="n">
         <v>119</v>
       </c>
-      <c r="E154" t="inlineStr">
+      <c r="E166" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4206,7 +4506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4219,14 +4519,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:25:49</t>
+          <t>Última actualización: 16:09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 28</t>
+          <t>Total filas: 31</t>
         </is>
       </c>
     </row>
@@ -4952,6 +5252,81 @@
         <v>109</v>
       </c>
       <c r="E33" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>16:09:00</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>17:15</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>66</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>16:09:00</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>17:45</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>96</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>16:09:00</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>17:55</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>106</v>
+      </c>
+      <c r="E36" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4968,7 +5343,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4981,14 +5356,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:25:49</t>
+          <t>Última actualización: 16:09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 28</t>
+          <t>Total filas: 29</t>
         </is>
       </c>
     </row>
@@ -5672,7 +6047,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>14:48:24</t>
+          <t>16:09:00</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -5686,7 +6061,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>102</v>
+        <v>21</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -5714,6 +6089,31 @@
         <v>117</v>
       </c>
       <c r="E33" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>16:09:00</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>17:23</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>74</v>
+      </c>
+      <c r="E34" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2180
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-03.xlsx
+++ b/data/horarios-141-2026-04-03.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E166"/>
+  <dimension ref="A1:E175"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:09:00</t>
+          <t>Última actualización: 16:50:18</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 161</t>
+          <t>Total filas: 170</t>
         </is>
       </c>
     </row>
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -558,7 +558,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -1058,7 +1058,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D29" t="n">
@@ -1083,7 +1083,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D30" t="n">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1333,7 +1333,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -3008,7 +3008,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -3033,7 +3033,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D108" t="n">
@@ -3423,7 +3423,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>14:01:59</t>
+          <t>14:48:24</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -3433,11 +3433,11 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>63</v>
+        <v>16</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>14:48:24</t>
+          <t>14:01:59</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>16</v>
+        <v>63</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -4173,7 +4173,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>16:09:00</t>
+          <t>16:50:18</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
@@ -4187,7 +4187,7 @@
         </is>
       </c>
       <c r="D154" t="n">
-        <v>42</v>
+        <v>1</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
@@ -4198,7 +4198,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>16:09:00</t>
+          <t>16:50:18</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
@@ -4212,7 +4212,7 @@
         </is>
       </c>
       <c r="D155" t="n">
-        <v>46</v>
+        <v>5</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
@@ -4248,7 +4248,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>16:09:00</t>
+          <t>16:50:18</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
@@ -4262,7 +4262,7 @@
         </is>
       </c>
       <c r="D157" t="n">
-        <v>56</v>
+        <v>15</v>
       </c>
       <c r="E157" t="inlineStr">
         <is>
@@ -4298,7 +4298,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>16:09:00</t>
+          <t>16:50:18</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -4312,7 +4312,7 @@
         </is>
       </c>
       <c r="D159" t="n">
-        <v>66</v>
+        <v>25</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4323,7 +4323,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>16:09:00</t>
+          <t>16:50:18</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -4337,7 +4337,7 @@
         </is>
       </c>
       <c r="D160" t="n">
-        <v>75</v>
+        <v>34</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4348,21 +4348,21 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>16:09:00</t>
+          <t>16:50:18</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>17:34</t>
+          <t>17:26</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D161" t="n">
-        <v>85</v>
+        <v>36</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4373,21 +4373,21 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>16:09:00</t>
+          <t>16:50:18</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>17:31</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D162" t="n">
-        <v>86</v>
+        <v>41</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
@@ -4403,16 +4403,16 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>17:38</t>
+          <t>17:34</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D163" t="n">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
@@ -4423,21 +4423,21 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>16:09:00</t>
+          <t>16:50:18</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>17:45</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D164" t="n">
-        <v>96</v>
+        <v>45</v>
       </c>
       <c r="E164" t="inlineStr">
         <is>
@@ -4448,21 +4448,21 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>16:09:00</t>
+          <t>16:50:18</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>17:55</t>
+          <t>17:37</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D165" t="n">
-        <v>106</v>
+        <v>47</v>
       </c>
       <c r="E165" t="inlineStr">
         <is>
@@ -4478,18 +4478,243 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
+          <t>17:38</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D166" t="n">
+        <v>89</v>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>16:50:18</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>17:45</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D167" t="n">
+        <v>55</v>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>16:50:18</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>17:55</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D168" t="n">
+        <v>65</v>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>16:50:18</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>18:04</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D169" t="n">
+        <v>74</v>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>16:09:00</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
           <t>18:08</t>
         </is>
       </c>
-      <c r="C166" t="inlineStr">
+      <c r="C170" t="inlineStr">
         <is>
           <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D166" t="n">
+      <c r="D170" t="n">
         <v>119</v>
       </c>
-      <c r="E166" t="inlineStr">
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>16:50:18</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D171" t="n">
+        <v>85</v>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>16:50:18</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>18:21</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D172" t="n">
+        <v>91</v>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>16:50:18</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>18:25</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D173" t="n">
+        <v>95</v>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>16:50:18</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>18:34</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D174" t="n">
+        <v>104</v>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>16:50:18</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>18:44</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D175" t="n">
+        <v>114</v>
+      </c>
+      <c r="E175" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4506,7 +4731,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4519,14 +4744,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:09:00</t>
+          <t>Última actualización: 16:50:18</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 31</t>
+          <t>Total filas: 32</t>
         </is>
       </c>
     </row>
@@ -4670,7 +4895,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -4695,7 +4920,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -5260,7 +5485,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>16:09:00</t>
+          <t>16:50:18</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -5274,7 +5499,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>66</v>
+        <v>25</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -5285,7 +5510,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>16:09:00</t>
+          <t>16:50:18</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -5299,7 +5524,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>96</v>
+        <v>55</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -5310,7 +5535,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>16:09:00</t>
+          <t>16:50:18</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -5324,9 +5549,34 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>106</v>
+        <v>65</v>
       </c>
       <c r="E36" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>16:50:18</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>85</v>
+      </c>
+      <c r="E37" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5343,7 +5593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5356,14 +5606,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:09:00</t>
+          <t>Última actualización: 16:50:18</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 29</t>
+          <t>Total filas: 30</t>
         </is>
       </c>
     </row>
@@ -6097,7 +6347,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>16:09:00</t>
+          <t>16:50:18</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -6111,9 +6361,34 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>74</v>
+        <v>33</v>
       </c>
       <c r="E34" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>16:50:18</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>115</v>
+      </c>
+      <c r="E35" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2181
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-03.xlsx
+++ b/data/horarios-141-2026-04-03.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E175"/>
+  <dimension ref="A1:E190"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:50:18</t>
+          <t>Última actualización: 17:18:54</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 170</t>
+          <t>Total filas: 185</t>
         </is>
       </c>
     </row>
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -558,7 +558,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -1108,7 +1108,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D31" t="n">
@@ -1133,7 +1133,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1333,7 +1333,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -3008,7 +3008,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -3033,7 +3033,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D108" t="n">
@@ -3423,7 +3423,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>14:48:24</t>
+          <t>14:01:59</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -3433,11 +3433,11 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>16</v>
+        <v>63</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>14:01:59</t>
+          <t>14:48:24</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>63</v>
+        <v>16</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -4323,12 +4323,12 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>16:50:18</t>
+          <t>17:18:54</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>17:24</t>
+          <t>17:18</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
@@ -4337,7 +4337,7 @@
         </is>
       </c>
       <c r="D160" t="n">
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4353,16 +4353,16 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>17:26</t>
+          <t>17:24</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D161" t="n">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4378,16 +4378,16 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>17:31</t>
+          <t>17:26</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D162" t="n">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
@@ -4398,12 +4398,12 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>16:09:00</t>
+          <t>17:18:54</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>17:34</t>
+          <t>17:31</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
@@ -4412,7 +4412,7 @@
         </is>
       </c>
       <c r="D163" t="n">
-        <v>85</v>
+        <v>13</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
@@ -4423,21 +4423,21 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>16:50:18</t>
+          <t>16:09:00</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>17:34</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D164" t="n">
-        <v>45</v>
+        <v>85</v>
       </c>
       <c r="E164" t="inlineStr">
         <is>
@@ -4448,21 +4448,21 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>16:50:18</t>
+          <t>17:18:54</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>17:37</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D165" t="n">
-        <v>47</v>
+        <v>17</v>
       </c>
       <c r="E165" t="inlineStr">
         <is>
@@ -4473,12 +4473,12 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>16:09:00</t>
+          <t>17:18:54</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>17:38</t>
+          <t>17:36</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
@@ -4487,7 +4487,7 @@
         </is>
       </c>
       <c r="D166" t="n">
-        <v>89</v>
+        <v>18</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
@@ -4503,16 +4503,16 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>17:45</t>
+          <t>17:37</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D167" t="n">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -4523,21 +4523,21 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>16:50:18</t>
+          <t>16:09:00</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>17:55</t>
+          <t>17:38</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D168" t="n">
-        <v>65</v>
+        <v>89</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
@@ -4548,21 +4548,21 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>16:50:18</t>
+          <t>17:18:54</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>18:04</t>
+          <t>17:44</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D169" t="n">
-        <v>74</v>
+        <v>26</v>
       </c>
       <c r="E169" t="inlineStr">
         <is>
@@ -4573,21 +4573,21 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>16:09:00</t>
+          <t>16:50:18</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>18:08</t>
+          <t>17:45</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D170" t="n">
-        <v>119</v>
+        <v>55</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
@@ -4598,21 +4598,21 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>16:50:18</t>
+          <t>17:18:54</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>18:15</t>
+          <t>17:54</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D171" t="n">
-        <v>85</v>
+        <v>36</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -4628,16 +4628,16 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>18:21</t>
+          <t>17:55</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D172" t="n">
-        <v>91</v>
+        <v>65</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -4648,21 +4648,21 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>16:50:18</t>
+          <t>17:18:54</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>18:25</t>
+          <t>18:03</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D173" t="n">
-        <v>95</v>
+        <v>45</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
@@ -4678,16 +4678,16 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>18:34</t>
+          <t>18:04</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D174" t="n">
-        <v>104</v>
+        <v>74</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -4698,23 +4698,398 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
+          <t>16:09:00</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>18:08</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D175" t="n">
+        <v>119</v>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>17:18:54</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>18:14</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D176" t="n">
+        <v>56</v>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
           <t>16:50:18</t>
         </is>
       </c>
-      <c r="B175" t="inlineStr">
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D177" t="n">
+        <v>85</v>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>17:18:54</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>18:17</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D178" t="n">
+        <v>59</v>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>16:50:18</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>18:21</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D179" t="n">
+        <v>91</v>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>17:18:54</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>18:24</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D180" t="n">
+        <v>66</v>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>16:50:18</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>18:25</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D181" t="n">
+        <v>95</v>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>17:18:54</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>18:34</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D182" t="n">
+        <v>76</v>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>17:18:54</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>18:36</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D183" t="n">
+        <v>78</v>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>17:18:54</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>18:43</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D184" t="n">
+        <v>85</v>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>16:50:18</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
         <is>
           <t>18:44</t>
         </is>
       </c>
-      <c r="C175" t="inlineStr">
+      <c r="C185" t="inlineStr">
         <is>
           <t>10_OLMOS</t>
         </is>
       </c>
-      <c r="D175" t="n">
+      <c r="D185" t="n">
         <v>114</v>
       </c>
-      <c r="E175" t="inlineStr">
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>17:18:54</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>18:54</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D186" t="n">
+        <v>96</v>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>17:18:54</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>18:59</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D187" t="n">
+        <v>101</v>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>17:18:54</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>19:04</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D188" t="n">
+        <v>106</v>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>17:18:54</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>19:16</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D189" t="n">
+        <v>118</v>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>17:18:54</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>19:16</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D190" t="n">
+        <v>118</v>
+      </c>
+      <c r="E190" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4731,7 +5106,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4744,14 +5119,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:50:18</t>
+          <t>Última actualización: 17:18:54</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 32</t>
+          <t>Total filas: 36</t>
         </is>
       </c>
     </row>
@@ -5510,12 +5885,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>16:50:18</t>
+          <t>17:18:54</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>17:45</t>
+          <t>17:44</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -5524,7 +5899,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>55</v>
+        <v>26</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -5540,16 +5915,16 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>17:55</t>
+          <t>17:45</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -5560,23 +5935,123 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
+          <t>17:18:54</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>17:54</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>36</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
           <t>16:50:18</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>17:55</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>65</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>17:18:54</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>18:14</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>56</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>16:50:18</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
         <is>
           <t>18:15</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C40" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D37" t="n">
+      <c r="D40" t="n">
         <v>85</v>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>17:18:54</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>18:59</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>101</v>
+      </c>
+      <c r="E41" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5593,7 +6068,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5606,14 +6081,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:50:18</t>
+          <t>Última actualización: 17:18:54</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 30</t>
+          <t>Total filas: 32</t>
         </is>
       </c>
     </row>
@@ -6322,7 +6797,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>15:25:49</t>
+          <t>17:18:54</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -6336,7 +6811,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>117</v>
+        <v>4</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -6372,25 +6847,75 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
+          <t>17:18:54</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>18:44</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>86</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
           <t>16:50:18</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B36" t="inlineStr">
         <is>
           <t>18:45</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C36" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D35" t="n">
+      <c r="D36" t="n">
         <v>115</v>
       </c>
-      <c r="E35" t="inlineStr">
+      <c r="E36" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>17:18:54</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>19:14</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>116</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2182
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-03.xlsx
+++ b/data/horarios-141-2026-04-03.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E190"/>
+  <dimension ref="A1:E195"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:18:54</t>
+          <t>Última actualización: 17:55:38</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 185</t>
+          <t>Total filas: 190</t>
         </is>
       </c>
     </row>
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -558,7 +558,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -1058,7 +1058,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D29" t="n">
@@ -1083,7 +1083,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D30" t="n">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1333,7 +1333,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -3008,7 +3008,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -3033,7 +3033,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D108" t="n">
@@ -3208,7 +3208,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D115" t="n">
@@ -3233,7 +3233,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D116" t="n">
@@ -4623,7 +4623,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>16:50:18</t>
+          <t>17:55:38</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="D172" t="n">
-        <v>65</v>
+        <v>0</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -4673,7 +4673,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>16:50:18</t>
+          <t>17:55:38</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
@@ -4687,7 +4687,7 @@
         </is>
       </c>
       <c r="D174" t="n">
-        <v>74</v>
+        <v>9</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -4723,7 +4723,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>17:18:54</t>
+          <t>17:55:38</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
@@ -4737,7 +4737,7 @@
         </is>
       </c>
       <c r="D176" t="n">
-        <v>56</v>
+        <v>19</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -4798,7 +4798,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>16:50:18</t>
+          <t>17:55:38</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
@@ -4812,7 +4812,7 @@
         </is>
       </c>
       <c r="D179" t="n">
-        <v>91</v>
+        <v>26</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
@@ -4823,7 +4823,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>17:18:54</t>
+          <t>17:55:38</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
@@ -4837,7 +4837,7 @@
         </is>
       </c>
       <c r="D180" t="n">
-        <v>66</v>
+        <v>29</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -4873,7 +4873,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>17:18:54</t>
+          <t>17:55:38</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
@@ -4887,7 +4887,7 @@
         </is>
       </c>
       <c r="D182" t="n">
-        <v>76</v>
+        <v>39</v>
       </c>
       <c r="E182" t="inlineStr">
         <is>
@@ -4898,7 +4898,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>17:18:54</t>
+          <t>17:55:38</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -4912,7 +4912,7 @@
         </is>
       </c>
       <c r="D183" t="n">
-        <v>78</v>
+        <v>41</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4948,7 +4948,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>16:50:18</t>
+          <t>17:55:38</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -4962,7 +4962,7 @@
         </is>
       </c>
       <c r="D185" t="n">
-        <v>114</v>
+        <v>49</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4973,7 +4973,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>17:18:54</t>
+          <t>17:55:38</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -4987,7 +4987,7 @@
         </is>
       </c>
       <c r="D186" t="n">
-        <v>96</v>
+        <v>59</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -4998,7 +4998,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>17:18:54</t>
+          <t>17:55:38</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -5012,7 +5012,7 @@
         </is>
       </c>
       <c r="D187" t="n">
-        <v>101</v>
+        <v>64</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -5023,7 +5023,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>17:18:54</t>
+          <t>17:55:38</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -5037,7 +5037,7 @@
         </is>
       </c>
       <c r="D188" t="n">
-        <v>106</v>
+        <v>69</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5048,7 +5048,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>17:18:54</t>
+          <t>17:55:38</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
@@ -5058,11 +5058,11 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D189" t="n">
-        <v>118</v>
+        <v>81</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -5073,7 +5073,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>17:18:54</t>
+          <t>17:55:38</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
@@ -5083,13 +5083,138 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D190" t="n">
-        <v>118</v>
+        <v>81</v>
       </c>
       <c r="E190" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>17:55:38</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>19:19</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D191" t="n">
+        <v>84</v>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>17:55:38</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>19:24</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D192" t="n">
+        <v>89</v>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>17:55:38</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>19:24</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D193" t="n">
+        <v>89</v>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>17:55:38</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>19:49</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D194" t="n">
+        <v>114</v>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>17:55:38</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>19:50</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D195" t="n">
+        <v>115</v>
+      </c>
+      <c r="E195" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5106,7 +5231,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5119,14 +5244,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:18:54</t>
+          <t>Última actualización: 17:55:38</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 36</t>
+          <t>Total filas: 37</t>
         </is>
       </c>
     </row>
@@ -5960,7 +6085,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>16:50:18</t>
+          <t>17:55:38</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -5974,7 +6099,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>65</v>
+        <v>0</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -5985,7 +6110,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>17:18:54</t>
+          <t>17:55:38</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -5999,7 +6124,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>56</v>
+        <v>19</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -6035,7 +6160,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>17:18:54</t>
+          <t>17:55:38</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -6049,9 +6174,34 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>101</v>
+        <v>64</v>
       </c>
       <c r="E41" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>17:55:38</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>19:24</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>89</v>
+      </c>
+      <c r="E42" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6068,7 +6218,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6081,14 +6231,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:18:54</t>
+          <t>Última actualización: 17:55:38</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 32</t>
+          <t>Total filas: 33</t>
         </is>
       </c>
     </row>
@@ -6847,7 +6997,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>17:18:54</t>
+          <t>17:55:38</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -6861,7 +7011,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>86</v>
+        <v>49</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -6897,7 +7047,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>17:18:54</t>
+          <t>17:55:38</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -6911,11 +7061,36 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>116</v>
+        <v>79</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>17:55:38</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>19:46</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>111</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2183
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-03.xlsx
+++ b/data/horarios-141-2026-04-03.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E195"/>
+  <dimension ref="A1:E204"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:55:38</t>
+          <t>Última actualización: 18:23:12</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 190</t>
+          <t>Total filas: 199</t>
         </is>
       </c>
     </row>
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -558,7 +558,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -1058,7 +1058,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D29" t="n">
@@ -1083,7 +1083,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D30" t="n">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1333,7 +1333,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -3008,7 +3008,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -3033,7 +3033,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D108" t="n">
@@ -3423,7 +3423,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>14:01:59</t>
+          <t>14:48:24</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -3433,11 +3433,11 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>63</v>
+        <v>16</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>14:48:24</t>
+          <t>14:01:59</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>16</v>
+        <v>63</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3798,7 +3798,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>15:25:49</t>
+          <t>14:01:59</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -3808,11 +3808,11 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D139" t="n">
-        <v>30</v>
+        <v>114</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -3823,7 +3823,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>14:01:59</t>
+          <t>15:25:49</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -3833,11 +3833,11 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D140" t="n">
-        <v>114</v>
+        <v>30</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
@@ -4823,7 +4823,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>17:55:38</t>
+          <t>18:23:11</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
@@ -4833,11 +4833,11 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D180" t="n">
-        <v>29</v>
+        <v>1</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -4848,12 +4848,12 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>16:50:18</t>
+          <t>17:55:38</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>18:25</t>
+          <t>18:24</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
@@ -4862,7 +4862,7 @@
         </is>
       </c>
       <c r="D181" t="n">
-        <v>95</v>
+        <v>29</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -4873,21 +4873,21 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>17:55:38</t>
+          <t>16:50:18</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>18:34</t>
+          <t>18:25</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D182" t="n">
-        <v>39</v>
+        <v>95</v>
       </c>
       <c r="E182" t="inlineStr">
         <is>
@@ -4898,21 +4898,21 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>17:55:38</t>
+          <t>18:23:11</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>18:36</t>
+          <t>18:26</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>41</v>
+        <v>3</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4923,21 +4923,21 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>17:18:54</t>
+          <t>18:23:11</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>18:43</t>
+          <t>18:34</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>85</v>
+        <v>11</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -4948,21 +4948,21 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>17:55:38</t>
+          <t>18:23:11</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>18:44</t>
+          <t>18:36</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>49</v>
+        <v>13</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4973,21 +4973,21 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>17:55:38</t>
+          <t>17:18:54</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>18:54</t>
+          <t>18:43</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>59</v>
+        <v>85</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -4998,21 +4998,21 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>17:55:38</t>
+          <t>18:23:11</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>18:59</t>
+          <t>18:44</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D187" t="n">
-        <v>64</v>
+        <v>21</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -5023,21 +5023,21 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>17:55:38</t>
+          <t>18:23:11</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>19:04</t>
+          <t>18:54</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D188" t="n">
-        <v>69</v>
+        <v>31</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5053,16 +5053,16 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>19:16</t>
+          <t>18:59</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D189" t="n">
-        <v>81</v>
+        <v>64</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -5073,21 +5073,21 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>17:55:38</t>
+          <t>18:23:11</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>19:16</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D190" t="n">
-        <v>81</v>
+        <v>37</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
@@ -5103,16 +5103,16 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>19:19</t>
+          <t>19:04</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D191" t="n">
-        <v>84</v>
+        <v>69</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -5128,16 +5128,16 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>19:24</t>
+          <t>19:16</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D192" t="n">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -5153,16 +5153,16 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>19:24</t>
+          <t>19:16</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5173,21 +5173,21 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>17:55:38</t>
+          <t>18:23:11</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>19:49</t>
+          <t>19:17</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D194" t="n">
-        <v>114</v>
+        <v>54</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
@@ -5203,18 +5203,243 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
+          <t>19:19</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D195" t="n">
+        <v>84</v>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>18:23:11</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>19:24</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D196" t="n">
+        <v>61</v>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>18:23:11</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>19:24</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D197" t="n">
+        <v>61</v>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>17:55:38</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>19:24</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D198" t="n">
+        <v>89</v>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>18:23:11</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>19:25</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D199" t="n">
+        <v>62</v>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>18:23:11</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>19:49</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D200" t="n">
+        <v>86</v>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>18:23:11</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
           <t>19:50</t>
         </is>
       </c>
-      <c r="C195" t="inlineStr">
+      <c r="C201" t="inlineStr">
         <is>
           <t>81_EL PELIGRO</t>
         </is>
       </c>
-      <c r="D195" t="n">
-        <v>115</v>
-      </c>
-      <c r="E195" t="inlineStr">
+      <c r="D201" t="n">
+        <v>87</v>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>18:23:11</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>19:56</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D202" t="n">
+        <v>93</v>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>18:23:11</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D203" t="n">
+        <v>112</v>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>18:23:11</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>20:16</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D204" t="n">
+        <v>113</v>
+      </c>
+      <c r="E204" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5231,7 +5456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5244,14 +5469,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:55:38</t>
+          <t>Última actualización: 18:23:12</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 37</t>
+          <t>Total filas: 40</t>
         </is>
       </c>
     </row>
@@ -6185,23 +6410,98 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
+          <t>18:23:11</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>37</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
           <t>17:55:38</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="B43" t="inlineStr">
         <is>
           <t>19:24</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C43" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D42" t="n">
+      <c r="D43" t="n">
         <v>89</v>
       </c>
-      <c r="E42" t="inlineStr">
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>18:23:11</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>19:25</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>62</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>18:23:11</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>112</v>
+      </c>
+      <c r="E45" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6218,7 +6518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E38"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6231,14 +6531,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:55:38</t>
+          <t>Última actualización: 18:23:12</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 33</t>
+          <t>Total filas: 35</t>
         </is>
       </c>
     </row>
@@ -7022,7 +7322,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>16:50:18</t>
+          <t>18:23:11</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -7036,7 +7336,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>115</v>
+        <v>22</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -7072,23 +7372,73 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
+          <t>18:23:11</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>19:15</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>52</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
           <t>17:55:38</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="B39" t="inlineStr">
         <is>
           <t>19:46</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C39" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D38" t="n">
+      <c r="D39" t="n">
         <v>111</v>
       </c>
-      <c r="E38" t="inlineStr">
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>18:23:11</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>19:47</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>84</v>
+      </c>
+      <c r="E40" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2184
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-03.xlsx
+++ b/data/horarios-141-2026-04-03.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E204"/>
+  <dimension ref="A1:E213"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:23:12</t>
+          <t>Última actualización: 18:53:58</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 199</t>
+          <t>Total filas: 208</t>
         </is>
       </c>
     </row>
@@ -1058,7 +1058,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D29" t="n">
@@ -1083,7 +1083,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D30" t="n">
@@ -1108,7 +1108,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D31" t="n">
@@ -1133,7 +1133,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -3008,7 +3008,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -3033,7 +3033,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D108" t="n">
@@ -3208,7 +3208,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D115" t="n">
@@ -3233,7 +3233,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D116" t="n">
@@ -3423,7 +3423,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>14:48:24</t>
+          <t>14:01:59</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -3433,11 +3433,11 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>16</v>
+        <v>63</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>14:01:59</t>
+          <t>14:48:24</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>63</v>
+        <v>16</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -5023,12 +5023,12 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>18:23:11</t>
+          <t>18:53:58</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>18:54</t>
+          <t>18:53</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
@@ -5037,7 +5037,7 @@
         </is>
       </c>
       <c r="D188" t="n">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5048,21 +5048,21 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>17:55:38</t>
+          <t>18:23:11</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>18:59</t>
+          <t>18:54</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D189" t="n">
-        <v>64</v>
+        <v>31</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -5073,12 +5073,12 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>18:23:11</t>
+          <t>18:53:58</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>18:59</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
@@ -5087,7 +5087,7 @@
         </is>
       </c>
       <c r="D190" t="n">
-        <v>37</v>
+        <v>6</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
@@ -5098,21 +5098,21 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>17:55:38</t>
+          <t>18:23:11</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>19:04</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D191" t="n">
-        <v>69</v>
+        <v>37</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -5123,21 +5123,21 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>17:55:38</t>
+          <t>18:53:58</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>19:16</t>
+          <t>19:04</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D192" t="n">
-        <v>81</v>
+        <v>11</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -5148,21 +5148,21 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>17:55:38</t>
+          <t>18:53:58</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>19:16</t>
+          <t>19:11</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>81</v>
+        <v>18</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5173,21 +5173,21 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>18:23:11</t>
+          <t>18:53:58</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>19:17</t>
+          <t>19:16</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D194" t="n">
-        <v>54</v>
+        <v>23</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
@@ -5198,21 +5198,21 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>17:55:38</t>
+          <t>18:53:58</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>19:19</t>
+          <t>19:16</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D195" t="n">
-        <v>84</v>
+        <v>23</v>
       </c>
       <c r="E195" t="inlineStr">
         <is>
@@ -5228,16 +5228,16 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>19:24</t>
+          <t>19:17</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D196" t="n">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
@@ -5248,21 +5248,21 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>18:23:11</t>
+          <t>17:55:38</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>19:24</t>
+          <t>19:19</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D197" t="n">
-        <v>61</v>
+        <v>84</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -5273,21 +5273,21 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>17:55:38</t>
+          <t>18:53:58</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>19:24</t>
+          <t>19:23</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D198" t="n">
-        <v>89</v>
+        <v>30</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
@@ -5303,16 +5303,16 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>19:25</t>
+          <t>19:24</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D199" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E199" t="inlineStr">
         <is>
@@ -5328,16 +5328,16 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>19:49</t>
+          <t>19:24</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D200" t="n">
-        <v>86</v>
+        <v>61</v>
       </c>
       <c r="E200" t="inlineStr">
         <is>
@@ -5348,21 +5348,21 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>18:23:11</t>
+          <t>18:53:58</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>19:50</t>
+          <t>19:24</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D201" t="n">
-        <v>87</v>
+        <v>31</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5378,16 +5378,16 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>19:56</t>
+          <t>19:25</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D202" t="n">
-        <v>93</v>
+        <v>62</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
@@ -5398,21 +5398,21 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>18:23:11</t>
+          <t>18:53:58</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>19:48</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D203" t="n">
-        <v>112</v>
+        <v>55</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
@@ -5428,18 +5428,243 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
+          <t>19:49</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D204" t="n">
+        <v>86</v>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>18:53:58</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>19:50</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D205" t="n">
+        <v>57</v>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>18:53:58</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>19:56</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D206" t="n">
+        <v>63</v>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>18:53:58</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>20:08</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D207" t="n">
+        <v>75</v>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>18:53:58</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>20:14</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D208" t="n">
+        <v>81</v>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>18:23:11</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D209" t="n">
+        <v>112</v>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>18:53:58</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D210" t="n">
+        <v>82</v>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>18:23:11</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
           <t>20:16</t>
         </is>
       </c>
-      <c r="C204" t="inlineStr">
+      <c r="C211" t="inlineStr">
         <is>
           <t>14_ABASTO</t>
         </is>
       </c>
-      <c r="D204" t="n">
+      <c r="D211" t="n">
         <v>113</v>
       </c>
-      <c r="E204" t="inlineStr">
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>18:53:58</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>20:39</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D212" t="n">
+        <v>106</v>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>18:53:58</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>20:41</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D213" t="n">
+        <v>108</v>
+      </c>
+      <c r="E213" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5456,7 +5681,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:E47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5469,14 +5694,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:23:12</t>
+          <t>Última actualización: 18:53:58</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 40</t>
+          <t>Total filas: 42</t>
         </is>
       </c>
     </row>
@@ -6385,7 +6610,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>17:55:38</t>
+          <t>18:53:58</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -6399,7 +6624,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>64</v>
+        <v>6</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -6435,7 +6660,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>17:55:38</t>
+          <t>18:53:58</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -6449,7 +6674,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>89</v>
+        <v>31</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -6485,23 +6710,73 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
+          <t>18:53:58</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>20:14</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>81</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
           <t>18:23:11</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="B46" t="inlineStr">
         <is>
           <t>20:15</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="C46" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D45" t="n">
+      <c r="D46" t="n">
         <v>112</v>
       </c>
-      <c r="E45" t="inlineStr">
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>18:53:58</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>20:39</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>106</v>
+      </c>
+      <c r="E47" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6518,7 +6793,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6531,14 +6806,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:23:12</t>
+          <t>Última actualización: 18:53:58</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 35</t>
+          <t>Total filas: 36</t>
         </is>
       </c>
     </row>
@@ -7347,7 +7622,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>17:55:38</t>
+          <t>18:53:58</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -7361,7 +7636,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>79</v>
+        <v>21</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -7397,7 +7672,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>17:55:38</t>
+          <t>18:53:58</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -7411,7 +7686,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>111</v>
+        <v>53</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -7439,6 +7714,31 @@
         <v>84</v>
       </c>
       <c r="E40" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>18:53:58</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>20:39</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>106</v>
+      </c>
+      <c r="E41" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2185
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-03.xlsx
+++ b/data/horarios-141-2026-04-03.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E213"/>
+  <dimension ref="A1:E222"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:53:58</t>
+          <t>Última actualización: 19:21:28</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 208</t>
+          <t>Total filas: 217</t>
         </is>
       </c>
     </row>
@@ -1058,7 +1058,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D29" t="n">
@@ -1083,7 +1083,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D30" t="n">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1333,7 +1333,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -3798,7 +3798,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>14:01:59</t>
+          <t>15:25:49</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -3808,11 +3808,11 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D139" t="n">
-        <v>114</v>
+        <v>30</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -3823,7 +3823,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>15:25:49</t>
+          <t>14:01:59</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -3833,11 +3833,11 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D140" t="n">
-        <v>30</v>
+        <v>114</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
@@ -4823,7 +4823,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>18:23:11</t>
+          <t>17:55:38</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
@@ -4833,11 +4833,11 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D180" t="n">
-        <v>1</v>
+        <v>29</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -4848,7 +4848,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>17:55:38</t>
+          <t>18:23:11</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
@@ -4858,11 +4858,11 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D181" t="n">
-        <v>29</v>
+        <v>1</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -5183,7 +5183,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D194" t="n">
@@ -5208,7 +5208,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D195" t="n">
@@ -5273,12 +5273,12 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>18:53:58</t>
+          <t>19:21:28</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>19:23</t>
+          <t>19:21</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
@@ -5287,7 +5287,7 @@
         </is>
       </c>
       <c r="D198" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
@@ -5298,21 +5298,21 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>18:23:11</t>
+          <t>19:21:28</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>19:24</t>
+          <t>19:21</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D199" t="n">
-        <v>61</v>
+        <v>0</v>
       </c>
       <c r="E199" t="inlineStr">
         <is>
@@ -5323,12 +5323,12 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>18:23:11</t>
+          <t>18:53:58</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>19:24</t>
+          <t>19:23</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
@@ -5337,7 +5337,7 @@
         </is>
       </c>
       <c r="D200" t="n">
-        <v>61</v>
+        <v>30</v>
       </c>
       <c r="E200" t="inlineStr">
         <is>
@@ -5348,7 +5348,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>18:53:58</t>
+          <t>18:23:11</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -5358,11 +5358,11 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D201" t="n">
-        <v>31</v>
+        <v>61</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5378,16 +5378,16 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>19:25</t>
+          <t>19:24</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D202" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
@@ -5403,16 +5403,16 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>19:48</t>
+          <t>19:24</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D203" t="n">
-        <v>55</v>
+        <v>31</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
@@ -5423,21 +5423,21 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>18:23:11</t>
+          <t>19:21:28</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>19:49</t>
+          <t>19:25</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D204" t="n">
-        <v>86</v>
+        <v>4</v>
       </c>
       <c r="E204" t="inlineStr">
         <is>
@@ -5453,16 +5453,16 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>19:50</t>
+          <t>19:48</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D205" t="n">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E205" t="inlineStr">
         <is>
@@ -5473,21 +5473,21 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>18:53:58</t>
+          <t>19:21:28</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>19:56</t>
+          <t>19:49</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D206" t="n">
-        <v>63</v>
+        <v>28</v>
       </c>
       <c r="E206" t="inlineStr">
         <is>
@@ -5498,21 +5498,21 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>18:53:58</t>
+          <t>19:21:28</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>20:08</t>
+          <t>19:50</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D207" t="n">
-        <v>75</v>
+        <v>29</v>
       </c>
       <c r="E207" t="inlineStr">
         <is>
@@ -5523,21 +5523,21 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>18:53:58</t>
+          <t>19:21:28</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>20:14</t>
+          <t>19:56</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D208" t="n">
-        <v>81</v>
+        <v>35</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -5548,21 +5548,21 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>18:23:11</t>
+          <t>19:21:28</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>20:01</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D209" t="n">
-        <v>112</v>
+        <v>40</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
@@ -5578,16 +5578,16 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>20:08</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D210" t="n">
-        <v>82</v>
+        <v>75</v>
       </c>
       <c r="E210" t="inlineStr">
         <is>
@@ -5598,21 +5598,21 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>18:23:11</t>
+          <t>18:53:58</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>20:16</t>
+          <t>20:14</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D211" t="n">
-        <v>113</v>
+        <v>81</v>
       </c>
       <c r="E211" t="inlineStr">
         <is>
@@ -5623,21 +5623,21 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>18:53:58</t>
+          <t>19:21:28</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>20:39</t>
+          <t>20:15</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D212" t="n">
-        <v>106</v>
+        <v>54</v>
       </c>
       <c r="E212" t="inlineStr">
         <is>
@@ -5648,23 +5648,248 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
+          <t>19:21:28</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D213" t="n">
+        <v>54</v>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>19:21:28</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D214" t="n">
+        <v>54</v>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>18:23:11</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>20:16</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D215" t="n">
+        <v>113</v>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>19:21:28</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>20:39</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D216" t="n">
+        <v>78</v>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
           <t>18:53:58</t>
         </is>
       </c>
-      <c r="B213" t="inlineStr">
+      <c r="B217" t="inlineStr">
         <is>
           <t>20:41</t>
         </is>
       </c>
-      <c r="C213" t="inlineStr">
+      <c r="C217" t="inlineStr">
         <is>
           <t>15_ABASTO</t>
         </is>
       </c>
-      <c r="D213" t="n">
+      <c r="D217" t="n">
         <v>108</v>
       </c>
-      <c r="E213" t="inlineStr">
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>19:21:28</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>20:42</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D218" t="n">
+        <v>81</v>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>19:21:28</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>20:51</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D219" t="n">
+        <v>90</v>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>19:21:28</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>20:56</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D220" t="n">
+        <v>95</v>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>19:21:28</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>21:06</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D221" t="n">
+        <v>105</v>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>19:21:28</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>21:07</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D222" t="n">
+        <v>106</v>
+      </c>
+      <c r="E222" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5694,7 +5919,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:53:58</t>
+          <t>Última actualización: 19:21:28</t>
         </is>
       </c>
     </row>
@@ -6685,7 +6910,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>18:23:11</t>
+          <t>19:21:28</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -6699,7 +6924,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>62</v>
+        <v>4</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -6735,7 +6960,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>18:23:11</t>
+          <t>19:21:28</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -6749,7 +6974,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>112</v>
+        <v>54</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -6760,7 +6985,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>18:53:58</t>
+          <t>19:21:28</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -6774,7 +6999,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>106</v>
+        <v>78</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -6806,7 +7031,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:53:58</t>
+          <t>Última actualización: 19:21:28</t>
         </is>
       </c>
     </row>
@@ -7697,7 +7922,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>18:23:11</t>
+          <t>19:21:28</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -7711,7 +7936,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>84</v>
+        <v>26</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -7722,7 +7947,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>18:53:58</t>
+          <t>19:21:28</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -7736,7 +7961,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>106</v>
+        <v>78</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2186
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-03.xlsx
+++ b/data/horarios-141-2026-04-03.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E222"/>
+  <dimension ref="A1:E230"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:21:28</t>
+          <t>Última actualización: 19:57:54</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 217</t>
+          <t>Total filas: 225</t>
         </is>
       </c>
     </row>
@@ -1058,7 +1058,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D29" t="n">
@@ -1083,7 +1083,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D30" t="n">
@@ -5183,7 +5183,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D194" t="n">
@@ -5208,7 +5208,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D195" t="n">
@@ -5283,7 +5283,7 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D198" t="n">
@@ -5308,7 +5308,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D199" t="n">
@@ -5548,21 +5548,21 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>19:21:28</t>
+          <t>19:57:54</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>20:01</t>
+          <t>19:57</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D209" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
@@ -5573,12 +5573,12 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>18:53:58</t>
+          <t>19:57:54</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>20:08</t>
+          <t>20:01</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
@@ -5587,7 +5587,7 @@
         </is>
       </c>
       <c r="D210" t="n">
-        <v>75</v>
+        <v>4</v>
       </c>
       <c r="E210" t="inlineStr">
         <is>
@@ -5603,16 +5603,16 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>20:14</t>
+          <t>20:08</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D211" t="n">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="E211" t="inlineStr">
         <is>
@@ -5623,12 +5623,12 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>19:21:28</t>
+          <t>19:57:54</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>20:14</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
@@ -5637,7 +5637,7 @@
         </is>
       </c>
       <c r="D212" t="n">
-        <v>54</v>
+        <v>17</v>
       </c>
       <c r="E212" t="inlineStr">
         <is>
@@ -5658,7 +5658,7 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D213" t="n">
@@ -5683,7 +5683,7 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D214" t="n">
@@ -5698,21 +5698,21 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>18:23:11</t>
+          <t>19:21:28</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>20:16</t>
+          <t>20:15</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>113</v>
+        <v>54</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5723,21 +5723,21 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>19:21:28</t>
+          <t>18:23:11</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>20:39</t>
+          <t>20:16</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>78</v>
+        <v>113</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5748,21 +5748,21 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>18:53:58</t>
+          <t>19:57:54</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>20:41</t>
+          <t>20:17</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D217" t="n">
-        <v>108</v>
+        <v>20</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -5773,21 +5773,21 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>19:21:28</t>
+          <t>19:57:54</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>20:42</t>
+          <t>20:35</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D218" t="n">
-        <v>81</v>
+        <v>38</v>
       </c>
       <c r="E218" t="inlineStr">
         <is>
@@ -5798,21 +5798,21 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>19:21:28</t>
+          <t>19:57:54</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>20:51</t>
+          <t>20:39</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D219" t="n">
-        <v>90</v>
+        <v>42</v>
       </c>
       <c r="E219" t="inlineStr">
         <is>
@@ -5823,21 +5823,21 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>19:21:28</t>
+          <t>19:57:54</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>20:56</t>
+          <t>20:41</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D220" t="n">
-        <v>95</v>
+        <v>44</v>
       </c>
       <c r="E220" t="inlineStr">
         <is>
@@ -5853,16 +5853,16 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>21:06</t>
+          <t>20:42</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D221" t="n">
-        <v>105</v>
+        <v>81</v>
       </c>
       <c r="E221" t="inlineStr">
         <is>
@@ -5878,18 +5878,218 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
+          <t>20:51</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D222" t="n">
+        <v>90</v>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>19:57:54</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>20:56</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D223" t="n">
+        <v>59</v>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>19:57:54</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>21:05</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D224" t="n">
+        <v>68</v>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>19:57:54</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>21:05</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D225" t="n">
+        <v>68</v>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>19:57:54</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>21:06</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D226" t="n">
+        <v>69</v>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>19:21:28</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>21:06</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D227" t="n">
+        <v>105</v>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>19:21:28</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
           <t>21:07</t>
         </is>
       </c>
-      <c r="C222" t="inlineStr">
+      <c r="C228" t="inlineStr">
         <is>
           <t>15_ABASTO</t>
         </is>
       </c>
-      <c r="D222" t="n">
+      <c r="D228" t="n">
         <v>106</v>
       </c>
-      <c r="E222" t="inlineStr">
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>19:57:54</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>21:34</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D229" t="n">
+        <v>97</v>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>19:57:54</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>21:36</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D230" t="n">
+        <v>99</v>
+      </c>
+      <c r="E230" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5919,7 +6119,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:21:28</t>
+          <t>Última actualización: 19:57:54</t>
         </is>
       </c>
     </row>
@@ -6935,7 +7135,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>18:53:58</t>
+          <t>19:57:54</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -6949,7 +7149,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>81</v>
+        <v>17</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -6985,7 +7185,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>19:21:28</t>
+          <t>19:57:54</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -6999,7 +7199,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>78</v>
+        <v>42</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -7018,7 +7218,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7031,14 +7231,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:21:28</t>
+          <t>Última actualización: 19:57:54</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 36</t>
+          <t>Total filas: 38</t>
         </is>
       </c>
     </row>
@@ -7964,6 +8164,56 @@
         <v>78</v>
       </c>
       <c r="E41" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>19:57:54</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>20:41</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>44</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>19:57:54</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>21:31</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>94</v>
+      </c>
+      <c r="E43" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2187
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-03.xlsx
+++ b/data/horarios-141-2026-04-03.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E230"/>
+  <dimension ref="A1:E234"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:57:54</t>
+          <t>Última actualización: 20:29:53</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 225</t>
+          <t>Total filas: 229</t>
         </is>
       </c>
     </row>
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -558,7 +558,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -1058,7 +1058,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D29" t="n">
@@ -1083,7 +1083,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D30" t="n">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1333,7 +1333,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -5348,7 +5348,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>18:23:11</t>
+          <t>18:53:58</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -5358,11 +5358,11 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D201" t="n">
-        <v>61</v>
+        <v>31</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5398,7 +5398,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>18:53:58</t>
+          <t>18:23:11</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
@@ -5408,11 +5408,11 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D203" t="n">
-        <v>31</v>
+        <v>61</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
@@ -5658,7 +5658,7 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D213" t="n">
@@ -5708,7 +5708,7 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D215" t="n">
@@ -5773,7 +5773,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>19:57:54</t>
+          <t>20:29:53</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
@@ -5787,7 +5787,7 @@
         </is>
       </c>
       <c r="D218" t="n">
-        <v>38</v>
+        <v>6</v>
       </c>
       <c r="E218" t="inlineStr">
         <is>
@@ -5798,7 +5798,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>19:57:54</t>
+          <t>20:29:53</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
@@ -5812,7 +5812,7 @@
         </is>
       </c>
       <c r="D219" t="n">
-        <v>42</v>
+        <v>10</v>
       </c>
       <c r="E219" t="inlineStr">
         <is>
@@ -5823,7 +5823,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>19:57:54</t>
+          <t>20:29:53</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
@@ -5837,7 +5837,7 @@
         </is>
       </c>
       <c r="D220" t="n">
-        <v>44</v>
+        <v>12</v>
       </c>
       <c r="E220" t="inlineStr">
         <is>
@@ -5873,7 +5873,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>19:21:28</t>
+          <t>20:29:53</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
@@ -5887,7 +5887,7 @@
         </is>
       </c>
       <c r="D222" t="n">
-        <v>90</v>
+        <v>22</v>
       </c>
       <c r="E222" t="inlineStr">
         <is>
@@ -5898,7 +5898,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>19:57:54</t>
+          <t>20:29:53</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
@@ -5912,7 +5912,7 @@
         </is>
       </c>
       <c r="D223" t="n">
-        <v>59</v>
+        <v>27</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
@@ -5948,7 +5948,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>19:57:54</t>
+          <t>20:29:53</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
@@ -5962,7 +5962,7 @@
         </is>
       </c>
       <c r="D225" t="n">
-        <v>68</v>
+        <v>36</v>
       </c>
       <c r="E225" t="inlineStr">
         <is>
@@ -5973,7 +5973,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>19:57:54</t>
+          <t>19:21:28</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
@@ -5983,11 +5983,11 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D226" t="n">
-        <v>69</v>
+        <v>105</v>
       </c>
       <c r="E226" t="inlineStr">
         <is>
@@ -5998,7 +5998,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>19:21:28</t>
+          <t>20:29:53</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
@@ -6008,11 +6008,11 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D227" t="n">
-        <v>105</v>
+        <v>37</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -6048,7 +6048,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>19:57:54</t>
+          <t>20:29:53</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
@@ -6062,7 +6062,7 @@
         </is>
       </c>
       <c r="D229" t="n">
-        <v>97</v>
+        <v>65</v>
       </c>
       <c r="E229" t="inlineStr">
         <is>
@@ -6073,23 +6073,123 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>19:57:54</t>
+          <t>20:29:53</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
         <is>
+          <t>21:35</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D230" t="n">
+        <v>66</v>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>20:29:53</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
           <t>21:36</t>
         </is>
       </c>
-      <c r="C230" t="inlineStr">
+      <c r="C231" t="inlineStr">
         <is>
           <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
-      <c r="D230" t="n">
-        <v>99</v>
-      </c>
-      <c r="E230" t="inlineStr">
+      <c r="D231" t="n">
+        <v>67</v>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>20:29:53</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>21:45</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D232" t="n">
+        <v>76</v>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>20:29:53</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>21:58</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D233" t="n">
+        <v>89</v>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>20:29:53</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>22:25</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D234" t="n">
+        <v>116</v>
+      </c>
+      <c r="E234" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6119,7 +6219,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:57:54</t>
+          <t>Última actualización: 20:29:53</t>
         </is>
       </c>
     </row>
@@ -7185,7 +7285,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>19:57:54</t>
+          <t>20:29:53</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -7199,7 +7299,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>42</v>
+        <v>10</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -7218,7 +7318,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E43"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7231,14 +7331,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:57:54</t>
+          <t>Última actualización: 20:29:53</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 38</t>
+          <t>Total filas: 40</t>
         </is>
       </c>
     </row>
@@ -8197,25 +8297,75 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>19:57:54</t>
+          <t>20:29:53</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
+          <t>20:42</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>13</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>20:29:53</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
           <t>21:31</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C44" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D43" t="n">
-        <v>94</v>
-      </c>
-      <c r="E43" t="inlineStr">
+      <c r="D44" t="n">
+        <v>62</v>
+      </c>
+      <c r="E44" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>20:29:53</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>22:08</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>99</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2188
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-03.xlsx
+++ b/data/horarios-141-2026-04-03.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E234"/>
+  <dimension ref="A1:E245"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:29:53</t>
+          <t>Última actualización: 20:57:03</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 229</t>
+          <t>Total filas: 240</t>
         </is>
       </c>
     </row>
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -558,7 +558,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -1058,7 +1058,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D29" t="n">
@@ -1083,7 +1083,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D30" t="n">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1333,7 +1333,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -3008,7 +3008,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -3033,7 +3033,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D108" t="n">
@@ -3208,7 +3208,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D115" t="n">
@@ -3233,7 +3233,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D116" t="n">
@@ -3423,7 +3423,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>14:01:59</t>
+          <t>14:48:24</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -3433,11 +3433,11 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>63</v>
+        <v>16</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>14:48:24</t>
+          <t>14:01:59</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>16</v>
+        <v>63</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3798,7 +3798,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>15:25:49</t>
+          <t>14:01:59</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -3808,11 +3808,11 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D139" t="n">
-        <v>30</v>
+        <v>114</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -3823,7 +3823,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>14:01:59</t>
+          <t>15:25:49</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -3833,11 +3833,11 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D140" t="n">
-        <v>114</v>
+        <v>30</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
@@ -4823,7 +4823,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>17:55:38</t>
+          <t>18:23:11</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
@@ -4833,11 +4833,11 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D180" t="n">
-        <v>29</v>
+        <v>1</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -4848,7 +4848,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>18:23:11</t>
+          <t>17:55:38</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
@@ -4858,11 +4858,11 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D181" t="n">
-        <v>1</v>
+        <v>29</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -5183,7 +5183,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D194" t="n">
@@ -5208,7 +5208,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D195" t="n">
@@ -5923,21 +5923,21 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>19:57:54</t>
+          <t>20:57:02</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>21:05</t>
+          <t>20:57</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D224" t="n">
-        <v>68</v>
+        <v>0</v>
       </c>
       <c r="E224" t="inlineStr">
         <is>
@@ -5973,21 +5973,21 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>19:21:28</t>
+          <t>19:57:54</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>21:06</t>
+          <t>21:05</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D226" t="n">
-        <v>105</v>
+        <v>68</v>
       </c>
       <c r="E226" t="inlineStr">
         <is>
@@ -6023,21 +6023,21 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>19:21:28</t>
+          <t>20:57:02</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>21:07</t>
+          <t>21:06</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D228" t="n">
-        <v>106</v>
+        <v>9</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
@@ -6048,21 +6048,21 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>20:29:53</t>
+          <t>20:57:02</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>21:34</t>
+          <t>21:07</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D229" t="n">
-        <v>65</v>
+        <v>10</v>
       </c>
       <c r="E229" t="inlineStr">
         <is>
@@ -6073,21 +6073,21 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>20:29:53</t>
+          <t>20:57:02</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>21:35</t>
+          <t>21:34</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D230" t="n">
-        <v>66</v>
+        <v>37</v>
       </c>
       <c r="E230" t="inlineStr">
         <is>
@@ -6103,16 +6103,16 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>21:36</t>
+          <t>21:35</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D231" t="n">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E231" t="inlineStr">
         <is>
@@ -6123,21 +6123,21 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>20:29:53</t>
+          <t>20:57:02</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>21:45</t>
+          <t>21:36</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D232" t="n">
-        <v>76</v>
+        <v>39</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -6153,16 +6153,16 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>21:58</t>
+          <t>21:36</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D233" t="n">
-        <v>89</v>
+        <v>67</v>
       </c>
       <c r="E233" t="inlineStr">
         <is>
@@ -6173,23 +6173,298 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
+          <t>20:57:02</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>21:37</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D234" t="n">
+        <v>40</v>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>20:57:02</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>21:40</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D235" t="n">
+        <v>43</v>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
           <t>20:29:53</t>
         </is>
       </c>
-      <c r="B234" t="inlineStr">
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>21:45</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D236" t="n">
+        <v>76</v>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>20:29:53</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>21:58</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D237" t="n">
+        <v>89</v>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>20:57:02</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>21:59</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D238" t="n">
+        <v>62</v>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>20:57:02</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>22:07</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D239" t="n">
+        <v>70</v>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>20:29:53</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
         <is>
           <t>22:25</t>
         </is>
       </c>
-      <c r="C234" t="inlineStr">
+      <c r="C240" t="inlineStr">
         <is>
           <t>14_ABASTO</t>
         </is>
       </c>
-      <c r="D234" t="n">
+      <c r="D240" t="n">
         <v>116</v>
       </c>
-      <c r="E234" t="inlineStr">
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>20:57:02</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>22:26</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D241" t="n">
+        <v>89</v>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>20:57:02</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>22:37</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D242" t="n">
+        <v>100</v>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>20:57:02</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>22:39</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D243" t="n">
+        <v>102</v>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>20:57:02</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>22:41</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D244" t="n">
+        <v>104</v>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>20:57:02</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>22:56</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D245" t="n">
+        <v>119</v>
+      </c>
+      <c r="E245" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6206,7 +6481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E47"/>
+  <dimension ref="A1:E48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6219,14 +6494,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:29:53</t>
+          <t>Última actualización: 20:57:03</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 42</t>
+          <t>Total filas: 43</t>
         </is>
       </c>
     </row>
@@ -7302,6 +7577,31 @@
         <v>10</v>
       </c>
       <c r="E47" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>20:57:02</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>22:37</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>100</v>
+      </c>
+      <c r="E48" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7318,7 +7618,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:E47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7331,14 +7631,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:29:53</t>
+          <t>Última actualización: 20:57:03</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 40</t>
+          <t>Total filas: 42</t>
         </is>
       </c>
     </row>
@@ -8347,23 +8647,73 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
+          <t>20:57:02</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>21:32</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>35</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
           <t>20:29:53</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="B46" t="inlineStr">
         <is>
           <t>22:08</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="C46" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-40 Y 115</t>
         </is>
       </c>
-      <c r="D45" t="n">
+      <c r="D46" t="n">
         <v>99</v>
       </c>
-      <c r="E45" t="inlineStr">
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>20:57:02</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>22:09</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>72</v>
+      </c>
+      <c r="E47" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2189
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-03.xlsx
+++ b/data/horarios-141-2026-04-03.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E245"/>
+  <dimension ref="A1:E251"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:57:03</t>
+          <t>Última actualización: 22:29:10</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 240</t>
+          <t>Total filas: 246</t>
         </is>
       </c>
     </row>
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -558,7 +558,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -1058,7 +1058,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D29" t="n">
@@ -1083,7 +1083,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D30" t="n">
@@ -1108,7 +1108,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D31" t="n">
@@ -1133,7 +1133,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -3008,7 +3008,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -3033,7 +3033,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D108" t="n">
@@ -5348,7 +5348,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>18:53:58</t>
+          <t>18:23:11</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -5358,11 +5358,11 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D201" t="n">
-        <v>31</v>
+        <v>61</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5383,7 +5383,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D202" t="n">
@@ -5398,7 +5398,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>18:23:11</t>
+          <t>18:53:58</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
@@ -5408,11 +5408,11 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D203" t="n">
-        <v>61</v>
+        <v>31</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
@@ -5658,7 +5658,7 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D213" t="n">
@@ -5683,7 +5683,7 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D214" t="n">
@@ -5708,7 +5708,7 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D215" t="n">
@@ -5948,7 +5948,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>20:29:53</t>
+          <t>19:57:54</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
@@ -5958,11 +5958,11 @@
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D225" t="n">
-        <v>36</v>
+        <v>68</v>
       </c>
       <c r="E225" t="inlineStr">
         <is>
@@ -5973,7 +5973,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>19:57:54</t>
+          <t>20:29:53</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
@@ -5983,11 +5983,11 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D226" t="n">
-        <v>68</v>
+        <v>36</v>
       </c>
       <c r="E226" t="inlineStr">
         <is>
@@ -6123,7 +6123,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>20:57:02</t>
+          <t>20:29:53</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -6133,11 +6133,11 @@
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D232" t="n">
-        <v>39</v>
+        <v>67</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -6148,7 +6148,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>20:29:53</t>
+          <t>20:57:02</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
@@ -6158,11 +6158,11 @@
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D233" t="n">
-        <v>67</v>
+        <v>39</v>
       </c>
       <c r="E233" t="inlineStr">
         <is>
@@ -6373,21 +6373,21 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>20:57:02</t>
+          <t>22:29:09</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>22:37</t>
+          <t>22:35</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D242" t="n">
-        <v>100</v>
+        <v>6</v>
       </c>
       <c r="E242" t="inlineStr">
         <is>
@@ -6398,21 +6398,21 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>20:57:02</t>
+          <t>22:29:09</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>22:39</t>
+          <t>22:37</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D243" t="n">
-        <v>102</v>
+        <v>8</v>
       </c>
       <c r="E243" t="inlineStr">
         <is>
@@ -6428,16 +6428,16 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>22:41</t>
+          <t>22:39</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D244" t="n">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="E244" t="inlineStr">
         <is>
@@ -6453,18 +6453,168 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
+          <t>22:41</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D245" t="n">
+        <v>104</v>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>22:29:09</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>22:49</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D246" t="n">
+        <v>20</v>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>22:29:09</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
           <t>22:56</t>
         </is>
       </c>
-      <c r="C245" t="inlineStr">
+      <c r="C247" t="inlineStr">
         <is>
           <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D245" t="n">
-        <v>119</v>
-      </c>
-      <c r="E245" t="inlineStr">
+      <c r="D247" t="n">
+        <v>27</v>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>22:29:09</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>23:07</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D248" t="n">
+        <v>38</v>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>22:29:09</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>23:26</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D249" t="n">
+        <v>57</v>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>22:29:09</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>23:36</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D250" t="n">
+        <v>67</v>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>22:29:09</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>23:41</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D251" t="n">
+        <v>72</v>
+      </c>
+      <c r="E251" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6481,7 +6631,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E48"/>
+  <dimension ref="A1:E49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6494,14 +6644,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:57:03</t>
+          <t>Última actualización: 22:29:10</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 43</t>
+          <t>Total filas: 44</t>
         </is>
       </c>
     </row>
@@ -6645,7 +6795,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -6670,7 +6820,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -7585,7 +7735,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>20:57:02</t>
+          <t>22:29:09</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -7599,9 +7749,34 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>100</v>
+        <v>8</v>
       </c>
       <c r="E48" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>22:29:09</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>23:41</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>72</v>
+      </c>
+      <c r="E49" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7631,7 +7806,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:57:03</t>
+          <t>Última actualización: 22:29:10</t>
         </is>
       </c>
     </row>

</xml_diff>